<commit_message>
feat: calculate compounding from account returns
</commit_message>
<xml_diff>
--- a/交易管理系统.xlsx
+++ b/交易管理系统.xlsx
@@ -262,6 +262,11 @@
         <t>默认等于实际买入股数；本系统按一次卖出处理。</t>
       </text>
     </comment>
+    <comment ref="AE1" authorId="0" shapeId="0">
+      <text>
+        <t>实际盈亏金额÷买入时账户金额快照；用于账户口径统计与逐笔复利。</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -282,9 +287,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TradeRecords" displayName="TradeRecords" ref="A1:AD201" headerRowCount="1">
-  <autoFilter ref="A1:AD201"/>
-  <tableColumns count="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TradeRecords" displayName="TradeRecords" ref="A1:AE201" headerRowCount="1">
+  <autoFilter ref="A1:AE201"/>
+  <tableColumns count="31">
     <tableColumn id="1" name="交易编号"/>
     <tableColumn id="2" name="股票代码"/>
     <tableColumn id="3" name="买入时账户金额"/>
@@ -309,12 +314,13 @@
     <tableColumn id="22" name="期望止损比例"/>
     <tableColumn id="23" name="盈亏比"/>
     <tableColumn id="24" name="实际盈亏金额"/>
-    <tableColumn id="25" name="实际收益率"/>
-    <tableColumn id="26" name="与平均盈利比例差值"/>
+    <tableColumn id="25" name="单笔仓位收益率"/>
+    <tableColumn id="26" name="账户收益率与平均盈利率差值"/>
     <tableColumn id="27" name="持有天数"/>
     <tableColumn id="28" name="复利容许平均亏损上限"/>
     <tableColumn id="29" name="复利风险判断"/>
     <tableColumn id="30" name="交易打分评价"/>
+    <tableColumn id="31" name="实际账户收益率"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -639,7 +645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD201"/>
+  <dimension ref="A1:AE201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -672,6 +678,7 @@
     <col width="22" customWidth="1" min="28" max="28"/>
     <col width="18" customWidth="1" min="29" max="29"/>
     <col width="18" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -797,12 +804,12 @@
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>实际收益率</t>
+          <t>单笔仓位收益率</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
-          <t>与平均盈利比例差值</t>
+          <t>账户收益率与平均盈利率差值</t>
         </is>
       </c>
       <c r="AA1" s="1" t="inlineStr">
@@ -823,6 +830,11 @@
       <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>交易打分评价</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>实际账户收益率</t>
         </is>
       </c>
     </row>
@@ -877,7 +889,7 @@
         <v/>
       </c>
       <c r="Z2" s="7">
-        <f>IF(OR(Y2="",'多次统计数据'!$B$8=""),"",Y2-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE2="",'多次统计数据'!$B$8=""),"",AE2-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA2" s="10">
@@ -893,6 +905,10 @@
         <v/>
       </c>
       <c r="AD2" s="2" t="n"/>
+      <c r="AE2" s="7">
+        <f>IF(OR(X2="",C2="",C2&lt;=0),"",X2/C2)</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n"/>
@@ -945,7 +961,7 @@
         <v/>
       </c>
       <c r="Z3" s="7">
-        <f>IF(OR(Y3="",'多次统计数据'!$B$8=""),"",Y3-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE3="",'多次统计数据'!$B$8=""),"",AE3-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA3" s="10">
@@ -961,6 +977,10 @@
         <v/>
       </c>
       <c r="AD3" s="2" t="n"/>
+      <c r="AE3" s="7">
+        <f>IF(OR(X3="",C3="",C3&lt;=0),"",X3/C3)</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n"/>
@@ -1013,7 +1033,7 @@
         <v/>
       </c>
       <c r="Z4" s="7">
-        <f>IF(OR(Y4="",'多次统计数据'!$B$8=""),"",Y4-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE4="",'多次统计数据'!$B$8=""),"",AE4-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA4" s="10">
@@ -1029,6 +1049,10 @@
         <v/>
       </c>
       <c r="AD4" s="2" t="n"/>
+      <c r="AE4" s="7">
+        <f>IF(OR(X4="",C4="",C4&lt;=0),"",X4/C4)</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n"/>
@@ -1081,7 +1105,7 @@
         <v/>
       </c>
       <c r="Z5" s="7">
-        <f>IF(OR(Y5="",'多次统计数据'!$B$8=""),"",Y5-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE5="",'多次统计数据'!$B$8=""),"",AE5-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA5" s="10">
@@ -1097,6 +1121,10 @@
         <v/>
       </c>
       <c r="AD5" s="2" t="n"/>
+      <c r="AE5" s="7">
+        <f>IF(OR(X5="",C5="",C5&lt;=0),"",X5/C5)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n"/>
@@ -1149,7 +1177,7 @@
         <v/>
       </c>
       <c r="Z6" s="7">
-        <f>IF(OR(Y6="",'多次统计数据'!$B$8=""),"",Y6-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE6="",'多次统计数据'!$B$8=""),"",AE6-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA6" s="10">
@@ -1165,6 +1193,10 @@
         <v/>
       </c>
       <c r="AD6" s="2" t="n"/>
+      <c r="AE6" s="7">
+        <f>IF(OR(X6="",C6="",C6&lt;=0),"",X6/C6)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n"/>
@@ -1217,7 +1249,7 @@
         <v/>
       </c>
       <c r="Z7" s="7">
-        <f>IF(OR(Y7="",'多次统计数据'!$B$8=""),"",Y7-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE7="",'多次统计数据'!$B$8=""),"",AE7-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA7" s="10">
@@ -1233,6 +1265,10 @@
         <v/>
       </c>
       <c r="AD7" s="2" t="n"/>
+      <c r="AE7" s="7">
+        <f>IF(OR(X7="",C7="",C7&lt;=0),"",X7/C7)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n"/>
@@ -1285,7 +1321,7 @@
         <v/>
       </c>
       <c r="Z8" s="7">
-        <f>IF(OR(Y8="",'多次统计数据'!$B$8=""),"",Y8-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE8="",'多次统计数据'!$B$8=""),"",AE8-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA8" s="10">
@@ -1301,6 +1337,10 @@
         <v/>
       </c>
       <c r="AD8" s="2" t="n"/>
+      <c r="AE8" s="7">
+        <f>IF(OR(X8="",C8="",C8&lt;=0),"",X8/C8)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n"/>
@@ -1353,7 +1393,7 @@
         <v/>
       </c>
       <c r="Z9" s="7">
-        <f>IF(OR(Y9="",'多次统计数据'!$B$8=""),"",Y9-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE9="",'多次统计数据'!$B$8=""),"",AE9-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA9" s="10">
@@ -1369,6 +1409,10 @@
         <v/>
       </c>
       <c r="AD9" s="2" t="n"/>
+      <c r="AE9" s="7">
+        <f>IF(OR(X9="",C9="",C9&lt;=0),"",X9/C9)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n"/>
@@ -1421,7 +1465,7 @@
         <v/>
       </c>
       <c r="Z10" s="7">
-        <f>IF(OR(Y10="",'多次统计数据'!$B$8=""),"",Y10-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE10="",'多次统计数据'!$B$8=""),"",AE10-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA10" s="10">
@@ -1437,6 +1481,10 @@
         <v/>
       </c>
       <c r="AD10" s="2" t="n"/>
+      <c r="AE10" s="7">
+        <f>IF(OR(X10="",C10="",C10&lt;=0),"",X10/C10)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n"/>
@@ -1489,7 +1537,7 @@
         <v/>
       </c>
       <c r="Z11" s="7">
-        <f>IF(OR(Y11="",'多次统计数据'!$B$8=""),"",Y11-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE11="",'多次统计数据'!$B$8=""),"",AE11-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA11" s="10">
@@ -1505,6 +1553,10 @@
         <v/>
       </c>
       <c r="AD11" s="2" t="n"/>
+      <c r="AE11" s="7">
+        <f>IF(OR(X11="",C11="",C11&lt;=0),"",X11/C11)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n"/>
@@ -1557,7 +1609,7 @@
         <v/>
       </c>
       <c r="Z12" s="7">
-        <f>IF(OR(Y12="",'多次统计数据'!$B$8=""),"",Y12-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE12="",'多次统计数据'!$B$8=""),"",AE12-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA12" s="10">
@@ -1573,6 +1625,10 @@
         <v/>
       </c>
       <c r="AD12" s="2" t="n"/>
+      <c r="AE12" s="7">
+        <f>IF(OR(X12="",C12="",C12&lt;=0),"",X12/C12)</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n"/>
@@ -1625,7 +1681,7 @@
         <v/>
       </c>
       <c r="Z13" s="7">
-        <f>IF(OR(Y13="",'多次统计数据'!$B$8=""),"",Y13-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE13="",'多次统计数据'!$B$8=""),"",AE13-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA13" s="10">
@@ -1641,6 +1697,10 @@
         <v/>
       </c>
       <c r="AD13" s="2" t="n"/>
+      <c r="AE13" s="7">
+        <f>IF(OR(X13="",C13="",C13&lt;=0),"",X13/C13)</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n"/>
@@ -1693,7 +1753,7 @@
         <v/>
       </c>
       <c r="Z14" s="7">
-        <f>IF(OR(Y14="",'多次统计数据'!$B$8=""),"",Y14-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE14="",'多次统计数据'!$B$8=""),"",AE14-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA14" s="10">
@@ -1709,6 +1769,10 @@
         <v/>
       </c>
       <c r="AD14" s="2" t="n"/>
+      <c r="AE14" s="7">
+        <f>IF(OR(X14="",C14="",C14&lt;=0),"",X14/C14)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n"/>
@@ -1761,7 +1825,7 @@
         <v/>
       </c>
       <c r="Z15" s="7">
-        <f>IF(OR(Y15="",'多次统计数据'!$B$8=""),"",Y15-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE15="",'多次统计数据'!$B$8=""),"",AE15-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA15" s="10">
@@ -1777,6 +1841,10 @@
         <v/>
       </c>
       <c r="AD15" s="2" t="n"/>
+      <c r="AE15" s="7">
+        <f>IF(OR(X15="",C15="",C15&lt;=0),"",X15/C15)</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n"/>
@@ -1829,7 +1897,7 @@
         <v/>
       </c>
       <c r="Z16" s="7">
-        <f>IF(OR(Y16="",'多次统计数据'!$B$8=""),"",Y16-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE16="",'多次统计数据'!$B$8=""),"",AE16-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA16" s="10">
@@ -1845,6 +1913,10 @@
         <v/>
       </c>
       <c r="AD16" s="2" t="n"/>
+      <c r="AE16" s="7">
+        <f>IF(OR(X16="",C16="",C16&lt;=0),"",X16/C16)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n"/>
@@ -1897,7 +1969,7 @@
         <v/>
       </c>
       <c r="Z17" s="7">
-        <f>IF(OR(Y17="",'多次统计数据'!$B$8=""),"",Y17-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE17="",'多次统计数据'!$B$8=""),"",AE17-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA17" s="10">
@@ -1913,6 +1985,10 @@
         <v/>
       </c>
       <c r="AD17" s="2" t="n"/>
+      <c r="AE17" s="7">
+        <f>IF(OR(X17="",C17="",C17&lt;=0),"",X17/C17)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n"/>
@@ -1965,7 +2041,7 @@
         <v/>
       </c>
       <c r="Z18" s="7">
-        <f>IF(OR(Y18="",'多次统计数据'!$B$8=""),"",Y18-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE18="",'多次统计数据'!$B$8=""),"",AE18-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA18" s="10">
@@ -1981,6 +2057,10 @@
         <v/>
       </c>
       <c r="AD18" s="2" t="n"/>
+      <c r="AE18" s="7">
+        <f>IF(OR(X18="",C18="",C18&lt;=0),"",X18/C18)</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n"/>
@@ -2033,7 +2113,7 @@
         <v/>
       </c>
       <c r="Z19" s="7">
-        <f>IF(OR(Y19="",'多次统计数据'!$B$8=""),"",Y19-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE19="",'多次统计数据'!$B$8=""),"",AE19-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA19" s="10">
@@ -2049,6 +2129,10 @@
         <v/>
       </c>
       <c r="AD19" s="2" t="n"/>
+      <c r="AE19" s="7">
+        <f>IF(OR(X19="",C19="",C19&lt;=0),"",X19/C19)</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n"/>
@@ -2101,7 +2185,7 @@
         <v/>
       </c>
       <c r="Z20" s="7">
-        <f>IF(OR(Y20="",'多次统计数据'!$B$8=""),"",Y20-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE20="",'多次统计数据'!$B$8=""),"",AE20-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA20" s="10">
@@ -2117,6 +2201,10 @@
         <v/>
       </c>
       <c r="AD20" s="2" t="n"/>
+      <c r="AE20" s="7">
+        <f>IF(OR(X20="",C20="",C20&lt;=0),"",X20/C20)</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n"/>
@@ -2169,7 +2257,7 @@
         <v/>
       </c>
       <c r="Z21" s="7">
-        <f>IF(OR(Y21="",'多次统计数据'!$B$8=""),"",Y21-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE21="",'多次统计数据'!$B$8=""),"",AE21-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA21" s="10">
@@ -2185,6 +2273,10 @@
         <v/>
       </c>
       <c r="AD21" s="2" t="n"/>
+      <c r="AE21" s="7">
+        <f>IF(OR(X21="",C21="",C21&lt;=0),"",X21/C21)</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n"/>
@@ -2237,7 +2329,7 @@
         <v/>
       </c>
       <c r="Z22" s="7">
-        <f>IF(OR(Y22="",'多次统计数据'!$B$8=""),"",Y22-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE22="",'多次统计数据'!$B$8=""),"",AE22-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA22" s="10">
@@ -2253,6 +2345,10 @@
         <v/>
       </c>
       <c r="AD22" s="2" t="n"/>
+      <c r="AE22" s="7">
+        <f>IF(OR(X22="",C22="",C22&lt;=0),"",X22/C22)</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n"/>
@@ -2305,7 +2401,7 @@
         <v/>
       </c>
       <c r="Z23" s="7">
-        <f>IF(OR(Y23="",'多次统计数据'!$B$8=""),"",Y23-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE23="",'多次统计数据'!$B$8=""),"",AE23-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA23" s="10">
@@ -2321,6 +2417,10 @@
         <v/>
       </c>
       <c r="AD23" s="2" t="n"/>
+      <c r="AE23" s="7">
+        <f>IF(OR(X23="",C23="",C23&lt;=0),"",X23/C23)</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n"/>
@@ -2373,7 +2473,7 @@
         <v/>
       </c>
       <c r="Z24" s="7">
-        <f>IF(OR(Y24="",'多次统计数据'!$B$8=""),"",Y24-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE24="",'多次统计数据'!$B$8=""),"",AE24-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA24" s="10">
@@ -2389,6 +2489,10 @@
         <v/>
       </c>
       <c r="AD24" s="2" t="n"/>
+      <c r="AE24" s="7">
+        <f>IF(OR(X24="",C24="",C24&lt;=0),"",X24/C24)</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n"/>
@@ -2441,7 +2545,7 @@
         <v/>
       </c>
       <c r="Z25" s="7">
-        <f>IF(OR(Y25="",'多次统计数据'!$B$8=""),"",Y25-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE25="",'多次统计数据'!$B$8=""),"",AE25-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA25" s="10">
@@ -2457,6 +2561,10 @@
         <v/>
       </c>
       <c r="AD25" s="2" t="n"/>
+      <c r="AE25" s="7">
+        <f>IF(OR(X25="",C25="",C25&lt;=0),"",X25/C25)</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n"/>
@@ -2509,7 +2617,7 @@
         <v/>
       </c>
       <c r="Z26" s="7">
-        <f>IF(OR(Y26="",'多次统计数据'!$B$8=""),"",Y26-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE26="",'多次统计数据'!$B$8=""),"",AE26-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA26" s="10">
@@ -2525,6 +2633,10 @@
         <v/>
       </c>
       <c r="AD26" s="2" t="n"/>
+      <c r="AE26" s="7">
+        <f>IF(OR(X26="",C26="",C26&lt;=0),"",X26/C26)</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n"/>
@@ -2577,7 +2689,7 @@
         <v/>
       </c>
       <c r="Z27" s="7">
-        <f>IF(OR(Y27="",'多次统计数据'!$B$8=""),"",Y27-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE27="",'多次统计数据'!$B$8=""),"",AE27-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA27" s="10">
@@ -2593,6 +2705,10 @@
         <v/>
       </c>
       <c r="AD27" s="2" t="n"/>
+      <c r="AE27" s="7">
+        <f>IF(OR(X27="",C27="",C27&lt;=0),"",X27/C27)</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n"/>
@@ -2645,7 +2761,7 @@
         <v/>
       </c>
       <c r="Z28" s="7">
-        <f>IF(OR(Y28="",'多次统计数据'!$B$8=""),"",Y28-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE28="",'多次统计数据'!$B$8=""),"",AE28-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA28" s="10">
@@ -2661,6 +2777,10 @@
         <v/>
       </c>
       <c r="AD28" s="2" t="n"/>
+      <c r="AE28" s="7">
+        <f>IF(OR(X28="",C28="",C28&lt;=0),"",X28/C28)</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n"/>
@@ -2713,7 +2833,7 @@
         <v/>
       </c>
       <c r="Z29" s="7">
-        <f>IF(OR(Y29="",'多次统计数据'!$B$8=""),"",Y29-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE29="",'多次统计数据'!$B$8=""),"",AE29-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA29" s="10">
@@ -2729,6 +2849,10 @@
         <v/>
       </c>
       <c r="AD29" s="2" t="n"/>
+      <c r="AE29" s="7">
+        <f>IF(OR(X29="",C29="",C29&lt;=0),"",X29/C29)</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n"/>
@@ -2781,7 +2905,7 @@
         <v/>
       </c>
       <c r="Z30" s="7">
-        <f>IF(OR(Y30="",'多次统计数据'!$B$8=""),"",Y30-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE30="",'多次统计数据'!$B$8=""),"",AE30-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA30" s="10">
@@ -2797,6 +2921,10 @@
         <v/>
       </c>
       <c r="AD30" s="2" t="n"/>
+      <c r="AE30" s="7">
+        <f>IF(OR(X30="",C30="",C30&lt;=0),"",X30/C30)</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n"/>
@@ -2849,7 +2977,7 @@
         <v/>
       </c>
       <c r="Z31" s="7">
-        <f>IF(OR(Y31="",'多次统计数据'!$B$8=""),"",Y31-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE31="",'多次统计数据'!$B$8=""),"",AE31-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA31" s="10">
@@ -2865,6 +2993,10 @@
         <v/>
       </c>
       <c r="AD31" s="2" t="n"/>
+      <c r="AE31" s="7">
+        <f>IF(OR(X31="",C31="",C31&lt;=0),"",X31/C31)</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n"/>
@@ -2917,7 +3049,7 @@
         <v/>
       </c>
       <c r="Z32" s="7">
-        <f>IF(OR(Y32="",'多次统计数据'!$B$8=""),"",Y32-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE32="",'多次统计数据'!$B$8=""),"",AE32-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA32" s="10">
@@ -2933,6 +3065,10 @@
         <v/>
       </c>
       <c r="AD32" s="2" t="n"/>
+      <c r="AE32" s="7">
+        <f>IF(OR(X32="",C32="",C32&lt;=0),"",X32/C32)</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n"/>
@@ -2985,7 +3121,7 @@
         <v/>
       </c>
       <c r="Z33" s="7">
-        <f>IF(OR(Y33="",'多次统计数据'!$B$8=""),"",Y33-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE33="",'多次统计数据'!$B$8=""),"",AE33-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA33" s="10">
@@ -3001,6 +3137,10 @@
         <v/>
       </c>
       <c r="AD33" s="2" t="n"/>
+      <c r="AE33" s="7">
+        <f>IF(OR(X33="",C33="",C33&lt;=0),"",X33/C33)</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n"/>
@@ -3053,7 +3193,7 @@
         <v/>
       </c>
       <c r="Z34" s="7">
-        <f>IF(OR(Y34="",'多次统计数据'!$B$8=""),"",Y34-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE34="",'多次统计数据'!$B$8=""),"",AE34-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA34" s="10">
@@ -3069,6 +3209,10 @@
         <v/>
       </c>
       <c r="AD34" s="2" t="n"/>
+      <c r="AE34" s="7">
+        <f>IF(OR(X34="",C34="",C34&lt;=0),"",X34/C34)</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n"/>
@@ -3121,7 +3265,7 @@
         <v/>
       </c>
       <c r="Z35" s="7">
-        <f>IF(OR(Y35="",'多次统计数据'!$B$8=""),"",Y35-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE35="",'多次统计数据'!$B$8=""),"",AE35-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA35" s="10">
@@ -3137,6 +3281,10 @@
         <v/>
       </c>
       <c r="AD35" s="2" t="n"/>
+      <c r="AE35" s="7">
+        <f>IF(OR(X35="",C35="",C35&lt;=0),"",X35/C35)</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n"/>
@@ -3189,7 +3337,7 @@
         <v/>
       </c>
       <c r="Z36" s="7">
-        <f>IF(OR(Y36="",'多次统计数据'!$B$8=""),"",Y36-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE36="",'多次统计数据'!$B$8=""),"",AE36-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA36" s="10">
@@ -3205,6 +3353,10 @@
         <v/>
       </c>
       <c r="AD36" s="2" t="n"/>
+      <c r="AE36" s="7">
+        <f>IF(OR(X36="",C36="",C36&lt;=0),"",X36/C36)</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n"/>
@@ -3257,7 +3409,7 @@
         <v/>
       </c>
       <c r="Z37" s="7">
-        <f>IF(OR(Y37="",'多次统计数据'!$B$8=""),"",Y37-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE37="",'多次统计数据'!$B$8=""),"",AE37-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA37" s="10">
@@ -3273,6 +3425,10 @@
         <v/>
       </c>
       <c r="AD37" s="2" t="n"/>
+      <c r="AE37" s="7">
+        <f>IF(OR(X37="",C37="",C37&lt;=0),"",X37/C37)</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n"/>
@@ -3325,7 +3481,7 @@
         <v/>
       </c>
       <c r="Z38" s="7">
-        <f>IF(OR(Y38="",'多次统计数据'!$B$8=""),"",Y38-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE38="",'多次统计数据'!$B$8=""),"",AE38-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA38" s="10">
@@ -3341,6 +3497,10 @@
         <v/>
       </c>
       <c r="AD38" s="2" t="n"/>
+      <c r="AE38" s="7">
+        <f>IF(OR(X38="",C38="",C38&lt;=0),"",X38/C38)</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n"/>
@@ -3393,7 +3553,7 @@
         <v/>
       </c>
       <c r="Z39" s="7">
-        <f>IF(OR(Y39="",'多次统计数据'!$B$8=""),"",Y39-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE39="",'多次统计数据'!$B$8=""),"",AE39-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA39" s="10">
@@ -3409,6 +3569,10 @@
         <v/>
       </c>
       <c r="AD39" s="2" t="n"/>
+      <c r="AE39" s="7">
+        <f>IF(OR(X39="",C39="",C39&lt;=0),"",X39/C39)</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n"/>
@@ -3461,7 +3625,7 @@
         <v/>
       </c>
       <c r="Z40" s="7">
-        <f>IF(OR(Y40="",'多次统计数据'!$B$8=""),"",Y40-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE40="",'多次统计数据'!$B$8=""),"",AE40-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA40" s="10">
@@ -3477,6 +3641,10 @@
         <v/>
       </c>
       <c r="AD40" s="2" t="n"/>
+      <c r="AE40" s="7">
+        <f>IF(OR(X40="",C40="",C40&lt;=0),"",X40/C40)</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n"/>
@@ -3529,7 +3697,7 @@
         <v/>
       </c>
       <c r="Z41" s="7">
-        <f>IF(OR(Y41="",'多次统计数据'!$B$8=""),"",Y41-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE41="",'多次统计数据'!$B$8=""),"",AE41-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA41" s="10">
@@ -3545,6 +3713,10 @@
         <v/>
       </c>
       <c r="AD41" s="2" t="n"/>
+      <c r="AE41" s="7">
+        <f>IF(OR(X41="",C41="",C41&lt;=0),"",X41/C41)</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n"/>
@@ -3597,7 +3769,7 @@
         <v/>
       </c>
       <c r="Z42" s="7">
-        <f>IF(OR(Y42="",'多次统计数据'!$B$8=""),"",Y42-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE42="",'多次统计数据'!$B$8=""),"",AE42-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA42" s="10">
@@ -3613,6 +3785,10 @@
         <v/>
       </c>
       <c r="AD42" s="2" t="n"/>
+      <c r="AE42" s="7">
+        <f>IF(OR(X42="",C42="",C42&lt;=0),"",X42/C42)</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n"/>
@@ -3665,7 +3841,7 @@
         <v/>
       </c>
       <c r="Z43" s="7">
-        <f>IF(OR(Y43="",'多次统计数据'!$B$8=""),"",Y43-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE43="",'多次统计数据'!$B$8=""),"",AE43-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA43" s="10">
@@ -3681,6 +3857,10 @@
         <v/>
       </c>
       <c r="AD43" s="2" t="n"/>
+      <c r="AE43" s="7">
+        <f>IF(OR(X43="",C43="",C43&lt;=0),"",X43/C43)</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n"/>
@@ -3733,7 +3913,7 @@
         <v/>
       </c>
       <c r="Z44" s="7">
-        <f>IF(OR(Y44="",'多次统计数据'!$B$8=""),"",Y44-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE44="",'多次统计数据'!$B$8=""),"",AE44-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA44" s="10">
@@ -3749,6 +3929,10 @@
         <v/>
       </c>
       <c r="AD44" s="2" t="n"/>
+      <c r="AE44" s="7">
+        <f>IF(OR(X44="",C44="",C44&lt;=0),"",X44/C44)</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n"/>
@@ -3801,7 +3985,7 @@
         <v/>
       </c>
       <c r="Z45" s="7">
-        <f>IF(OR(Y45="",'多次统计数据'!$B$8=""),"",Y45-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE45="",'多次统计数据'!$B$8=""),"",AE45-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA45" s="10">
@@ -3817,6 +4001,10 @@
         <v/>
       </c>
       <c r="AD45" s="2" t="n"/>
+      <c r="AE45" s="7">
+        <f>IF(OR(X45="",C45="",C45&lt;=0),"",X45/C45)</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n"/>
@@ -3869,7 +4057,7 @@
         <v/>
       </c>
       <c r="Z46" s="7">
-        <f>IF(OR(Y46="",'多次统计数据'!$B$8=""),"",Y46-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE46="",'多次统计数据'!$B$8=""),"",AE46-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA46" s="10">
@@ -3885,6 +4073,10 @@
         <v/>
       </c>
       <c r="AD46" s="2" t="n"/>
+      <c r="AE46" s="7">
+        <f>IF(OR(X46="",C46="",C46&lt;=0),"",X46/C46)</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n"/>
@@ -3937,7 +4129,7 @@
         <v/>
       </c>
       <c r="Z47" s="7">
-        <f>IF(OR(Y47="",'多次统计数据'!$B$8=""),"",Y47-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE47="",'多次统计数据'!$B$8=""),"",AE47-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA47" s="10">
@@ -3953,6 +4145,10 @@
         <v/>
       </c>
       <c r="AD47" s="2" t="n"/>
+      <c r="AE47" s="7">
+        <f>IF(OR(X47="",C47="",C47&lt;=0),"",X47/C47)</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n"/>
@@ -4005,7 +4201,7 @@
         <v/>
       </c>
       <c r="Z48" s="7">
-        <f>IF(OR(Y48="",'多次统计数据'!$B$8=""),"",Y48-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE48="",'多次统计数据'!$B$8=""),"",AE48-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA48" s="10">
@@ -4021,6 +4217,10 @@
         <v/>
       </c>
       <c r="AD48" s="2" t="n"/>
+      <c r="AE48" s="7">
+        <f>IF(OR(X48="",C48="",C48&lt;=0),"",X48/C48)</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n"/>
@@ -4073,7 +4273,7 @@
         <v/>
       </c>
       <c r="Z49" s="7">
-        <f>IF(OR(Y49="",'多次统计数据'!$B$8=""),"",Y49-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE49="",'多次统计数据'!$B$8=""),"",AE49-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA49" s="10">
@@ -4089,6 +4289,10 @@
         <v/>
       </c>
       <c r="AD49" s="2" t="n"/>
+      <c r="AE49" s="7">
+        <f>IF(OR(X49="",C49="",C49&lt;=0),"",X49/C49)</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n"/>
@@ -4141,7 +4345,7 @@
         <v/>
       </c>
       <c r="Z50" s="7">
-        <f>IF(OR(Y50="",'多次统计数据'!$B$8=""),"",Y50-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE50="",'多次统计数据'!$B$8=""),"",AE50-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA50" s="10">
@@ -4157,6 +4361,10 @@
         <v/>
       </c>
       <c r="AD50" s="2" t="n"/>
+      <c r="AE50" s="7">
+        <f>IF(OR(X50="",C50="",C50&lt;=0),"",X50/C50)</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n"/>
@@ -4209,7 +4417,7 @@
         <v/>
       </c>
       <c r="Z51" s="7">
-        <f>IF(OR(Y51="",'多次统计数据'!$B$8=""),"",Y51-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE51="",'多次统计数据'!$B$8=""),"",AE51-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA51" s="10">
@@ -4225,6 +4433,10 @@
         <v/>
       </c>
       <c r="AD51" s="2" t="n"/>
+      <c r="AE51" s="7">
+        <f>IF(OR(X51="",C51="",C51&lt;=0),"",X51/C51)</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n"/>
@@ -4277,7 +4489,7 @@
         <v/>
       </c>
       <c r="Z52" s="7">
-        <f>IF(OR(Y52="",'多次统计数据'!$B$8=""),"",Y52-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE52="",'多次统计数据'!$B$8=""),"",AE52-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA52" s="10">
@@ -4293,6 +4505,10 @@
         <v/>
       </c>
       <c r="AD52" s="2" t="n"/>
+      <c r="AE52" s="7">
+        <f>IF(OR(X52="",C52="",C52&lt;=0),"",X52/C52)</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n"/>
@@ -4345,7 +4561,7 @@
         <v/>
       </c>
       <c r="Z53" s="7">
-        <f>IF(OR(Y53="",'多次统计数据'!$B$8=""),"",Y53-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE53="",'多次统计数据'!$B$8=""),"",AE53-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA53" s="10">
@@ -4361,6 +4577,10 @@
         <v/>
       </c>
       <c r="AD53" s="2" t="n"/>
+      <c r="AE53" s="7">
+        <f>IF(OR(X53="",C53="",C53&lt;=0),"",X53/C53)</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n"/>
@@ -4413,7 +4633,7 @@
         <v/>
       </c>
       <c r="Z54" s="7">
-        <f>IF(OR(Y54="",'多次统计数据'!$B$8=""),"",Y54-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE54="",'多次统计数据'!$B$8=""),"",AE54-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA54" s="10">
@@ -4429,6 +4649,10 @@
         <v/>
       </c>
       <c r="AD54" s="2" t="n"/>
+      <c r="AE54" s="7">
+        <f>IF(OR(X54="",C54="",C54&lt;=0),"",X54/C54)</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n"/>
@@ -4481,7 +4705,7 @@
         <v/>
       </c>
       <c r="Z55" s="7">
-        <f>IF(OR(Y55="",'多次统计数据'!$B$8=""),"",Y55-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE55="",'多次统计数据'!$B$8=""),"",AE55-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA55" s="10">
@@ -4497,6 +4721,10 @@
         <v/>
       </c>
       <c r="AD55" s="2" t="n"/>
+      <c r="AE55" s="7">
+        <f>IF(OR(X55="",C55="",C55&lt;=0),"",X55/C55)</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n"/>
@@ -4549,7 +4777,7 @@
         <v/>
       </c>
       <c r="Z56" s="7">
-        <f>IF(OR(Y56="",'多次统计数据'!$B$8=""),"",Y56-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE56="",'多次统计数据'!$B$8=""),"",AE56-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA56" s="10">
@@ -4565,6 +4793,10 @@
         <v/>
       </c>
       <c r="AD56" s="2" t="n"/>
+      <c r="AE56" s="7">
+        <f>IF(OR(X56="",C56="",C56&lt;=0),"",X56/C56)</f>
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n"/>
@@ -4617,7 +4849,7 @@
         <v/>
       </c>
       <c r="Z57" s="7">
-        <f>IF(OR(Y57="",'多次统计数据'!$B$8=""),"",Y57-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE57="",'多次统计数据'!$B$8=""),"",AE57-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA57" s="10">
@@ -4633,6 +4865,10 @@
         <v/>
       </c>
       <c r="AD57" s="2" t="n"/>
+      <c r="AE57" s="7">
+        <f>IF(OR(X57="",C57="",C57&lt;=0),"",X57/C57)</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n"/>
@@ -4685,7 +4921,7 @@
         <v/>
       </c>
       <c r="Z58" s="7">
-        <f>IF(OR(Y58="",'多次统计数据'!$B$8=""),"",Y58-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE58="",'多次统计数据'!$B$8=""),"",AE58-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA58" s="10">
@@ -4701,6 +4937,10 @@
         <v/>
       </c>
       <c r="AD58" s="2" t="n"/>
+      <c r="AE58" s="7">
+        <f>IF(OR(X58="",C58="",C58&lt;=0),"",X58/C58)</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n"/>
@@ -4753,7 +4993,7 @@
         <v/>
       </c>
       <c r="Z59" s="7">
-        <f>IF(OR(Y59="",'多次统计数据'!$B$8=""),"",Y59-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE59="",'多次统计数据'!$B$8=""),"",AE59-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA59" s="10">
@@ -4769,6 +5009,10 @@
         <v/>
       </c>
       <c r="AD59" s="2" t="n"/>
+      <c r="AE59" s="7">
+        <f>IF(OR(X59="",C59="",C59&lt;=0),"",X59/C59)</f>
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n"/>
@@ -4821,7 +5065,7 @@
         <v/>
       </c>
       <c r="Z60" s="7">
-        <f>IF(OR(Y60="",'多次统计数据'!$B$8=""),"",Y60-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE60="",'多次统计数据'!$B$8=""),"",AE60-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA60" s="10">
@@ -4837,6 +5081,10 @@
         <v/>
       </c>
       <c r="AD60" s="2" t="n"/>
+      <c r="AE60" s="7">
+        <f>IF(OR(X60="",C60="",C60&lt;=0),"",X60/C60)</f>
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n"/>
@@ -4889,7 +5137,7 @@
         <v/>
       </c>
       <c r="Z61" s="7">
-        <f>IF(OR(Y61="",'多次统计数据'!$B$8=""),"",Y61-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE61="",'多次统计数据'!$B$8=""),"",AE61-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA61" s="10">
@@ -4905,6 +5153,10 @@
         <v/>
       </c>
       <c r="AD61" s="2" t="n"/>
+      <c r="AE61" s="7">
+        <f>IF(OR(X61="",C61="",C61&lt;=0),"",X61/C61)</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n"/>
@@ -4957,7 +5209,7 @@
         <v/>
       </c>
       <c r="Z62" s="7">
-        <f>IF(OR(Y62="",'多次统计数据'!$B$8=""),"",Y62-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE62="",'多次统计数据'!$B$8=""),"",AE62-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA62" s="10">
@@ -4973,6 +5225,10 @@
         <v/>
       </c>
       <c r="AD62" s="2" t="n"/>
+      <c r="AE62" s="7">
+        <f>IF(OR(X62="",C62="",C62&lt;=0),"",X62/C62)</f>
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n"/>
@@ -5025,7 +5281,7 @@
         <v/>
       </c>
       <c r="Z63" s="7">
-        <f>IF(OR(Y63="",'多次统计数据'!$B$8=""),"",Y63-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE63="",'多次统计数据'!$B$8=""),"",AE63-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA63" s="10">
@@ -5041,6 +5297,10 @@
         <v/>
       </c>
       <c r="AD63" s="2" t="n"/>
+      <c r="AE63" s="7">
+        <f>IF(OR(X63="",C63="",C63&lt;=0),"",X63/C63)</f>
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n"/>
@@ -5093,7 +5353,7 @@
         <v/>
       </c>
       <c r="Z64" s="7">
-        <f>IF(OR(Y64="",'多次统计数据'!$B$8=""),"",Y64-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE64="",'多次统计数据'!$B$8=""),"",AE64-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA64" s="10">
@@ -5109,6 +5369,10 @@
         <v/>
       </c>
       <c r="AD64" s="2" t="n"/>
+      <c r="AE64" s="7">
+        <f>IF(OR(X64="",C64="",C64&lt;=0),"",X64/C64)</f>
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n"/>
@@ -5161,7 +5425,7 @@
         <v/>
       </c>
       <c r="Z65" s="7">
-        <f>IF(OR(Y65="",'多次统计数据'!$B$8=""),"",Y65-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE65="",'多次统计数据'!$B$8=""),"",AE65-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA65" s="10">
@@ -5177,6 +5441,10 @@
         <v/>
       </c>
       <c r="AD65" s="2" t="n"/>
+      <c r="AE65" s="7">
+        <f>IF(OR(X65="",C65="",C65&lt;=0),"",X65/C65)</f>
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n"/>
@@ -5229,7 +5497,7 @@
         <v/>
       </c>
       <c r="Z66" s="7">
-        <f>IF(OR(Y66="",'多次统计数据'!$B$8=""),"",Y66-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE66="",'多次统计数据'!$B$8=""),"",AE66-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA66" s="10">
@@ -5245,6 +5513,10 @@
         <v/>
       </c>
       <c r="AD66" s="2" t="n"/>
+      <c r="AE66" s="7">
+        <f>IF(OR(X66="",C66="",C66&lt;=0),"",X66/C66)</f>
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n"/>
@@ -5297,7 +5569,7 @@
         <v/>
       </c>
       <c r="Z67" s="7">
-        <f>IF(OR(Y67="",'多次统计数据'!$B$8=""),"",Y67-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE67="",'多次统计数据'!$B$8=""),"",AE67-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA67" s="10">
@@ -5313,6 +5585,10 @@
         <v/>
       </c>
       <c r="AD67" s="2" t="n"/>
+      <c r="AE67" s="7">
+        <f>IF(OR(X67="",C67="",C67&lt;=0),"",X67/C67)</f>
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n"/>
@@ -5365,7 +5641,7 @@
         <v/>
       </c>
       <c r="Z68" s="7">
-        <f>IF(OR(Y68="",'多次统计数据'!$B$8=""),"",Y68-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE68="",'多次统计数据'!$B$8=""),"",AE68-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA68" s="10">
@@ -5381,6 +5657,10 @@
         <v/>
       </c>
       <c r="AD68" s="2" t="n"/>
+      <c r="AE68" s="7">
+        <f>IF(OR(X68="",C68="",C68&lt;=0),"",X68/C68)</f>
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n"/>
@@ -5433,7 +5713,7 @@
         <v/>
       </c>
       <c r="Z69" s="7">
-        <f>IF(OR(Y69="",'多次统计数据'!$B$8=""),"",Y69-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE69="",'多次统计数据'!$B$8=""),"",AE69-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA69" s="10">
@@ -5449,6 +5729,10 @@
         <v/>
       </c>
       <c r="AD69" s="2" t="n"/>
+      <c r="AE69" s="7">
+        <f>IF(OR(X69="",C69="",C69&lt;=0),"",X69/C69)</f>
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n"/>
@@ -5501,7 +5785,7 @@
         <v/>
       </c>
       <c r="Z70" s="7">
-        <f>IF(OR(Y70="",'多次统计数据'!$B$8=""),"",Y70-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE70="",'多次统计数据'!$B$8=""),"",AE70-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA70" s="10">
@@ -5517,6 +5801,10 @@
         <v/>
       </c>
       <c r="AD70" s="2" t="n"/>
+      <c r="AE70" s="7">
+        <f>IF(OR(X70="",C70="",C70&lt;=0),"",X70/C70)</f>
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n"/>
@@ -5569,7 +5857,7 @@
         <v/>
       </c>
       <c r="Z71" s="7">
-        <f>IF(OR(Y71="",'多次统计数据'!$B$8=""),"",Y71-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE71="",'多次统计数据'!$B$8=""),"",AE71-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA71" s="10">
@@ -5585,6 +5873,10 @@
         <v/>
       </c>
       <c r="AD71" s="2" t="n"/>
+      <c r="AE71" s="7">
+        <f>IF(OR(X71="",C71="",C71&lt;=0),"",X71/C71)</f>
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n"/>
@@ -5637,7 +5929,7 @@
         <v/>
       </c>
       <c r="Z72" s="7">
-        <f>IF(OR(Y72="",'多次统计数据'!$B$8=""),"",Y72-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE72="",'多次统计数据'!$B$8=""),"",AE72-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA72" s="10">
@@ -5653,6 +5945,10 @@
         <v/>
       </c>
       <c r="AD72" s="2" t="n"/>
+      <c r="AE72" s="7">
+        <f>IF(OR(X72="",C72="",C72&lt;=0),"",X72/C72)</f>
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n"/>
@@ -5705,7 +6001,7 @@
         <v/>
       </c>
       <c r="Z73" s="7">
-        <f>IF(OR(Y73="",'多次统计数据'!$B$8=""),"",Y73-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE73="",'多次统计数据'!$B$8=""),"",AE73-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA73" s="10">
@@ -5721,6 +6017,10 @@
         <v/>
       </c>
       <c r="AD73" s="2" t="n"/>
+      <c r="AE73" s="7">
+        <f>IF(OR(X73="",C73="",C73&lt;=0),"",X73/C73)</f>
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n"/>
@@ -5773,7 +6073,7 @@
         <v/>
       </c>
       <c r="Z74" s="7">
-        <f>IF(OR(Y74="",'多次统计数据'!$B$8=""),"",Y74-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE74="",'多次统计数据'!$B$8=""),"",AE74-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA74" s="10">
@@ -5789,6 +6089,10 @@
         <v/>
       </c>
       <c r="AD74" s="2" t="n"/>
+      <c r="AE74" s="7">
+        <f>IF(OR(X74="",C74="",C74&lt;=0),"",X74/C74)</f>
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n"/>
@@ -5841,7 +6145,7 @@
         <v/>
       </c>
       <c r="Z75" s="7">
-        <f>IF(OR(Y75="",'多次统计数据'!$B$8=""),"",Y75-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE75="",'多次统计数据'!$B$8=""),"",AE75-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA75" s="10">
@@ -5857,6 +6161,10 @@
         <v/>
       </c>
       <c r="AD75" s="2" t="n"/>
+      <c r="AE75" s="7">
+        <f>IF(OR(X75="",C75="",C75&lt;=0),"",X75/C75)</f>
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n"/>
@@ -5909,7 +6217,7 @@
         <v/>
       </c>
       <c r="Z76" s="7">
-        <f>IF(OR(Y76="",'多次统计数据'!$B$8=""),"",Y76-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE76="",'多次统计数据'!$B$8=""),"",AE76-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA76" s="10">
@@ -5925,6 +6233,10 @@
         <v/>
       </c>
       <c r="AD76" s="2" t="n"/>
+      <c r="AE76" s="7">
+        <f>IF(OR(X76="",C76="",C76&lt;=0),"",X76/C76)</f>
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n"/>
@@ -5977,7 +6289,7 @@
         <v/>
       </c>
       <c r="Z77" s="7">
-        <f>IF(OR(Y77="",'多次统计数据'!$B$8=""),"",Y77-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE77="",'多次统计数据'!$B$8=""),"",AE77-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA77" s="10">
@@ -5993,6 +6305,10 @@
         <v/>
       </c>
       <c r="AD77" s="2" t="n"/>
+      <c r="AE77" s="7">
+        <f>IF(OR(X77="",C77="",C77&lt;=0),"",X77/C77)</f>
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n"/>
@@ -6045,7 +6361,7 @@
         <v/>
       </c>
       <c r="Z78" s="7">
-        <f>IF(OR(Y78="",'多次统计数据'!$B$8=""),"",Y78-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE78="",'多次统计数据'!$B$8=""),"",AE78-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA78" s="10">
@@ -6061,6 +6377,10 @@
         <v/>
       </c>
       <c r="AD78" s="2" t="n"/>
+      <c r="AE78" s="7">
+        <f>IF(OR(X78="",C78="",C78&lt;=0),"",X78/C78)</f>
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n"/>
@@ -6113,7 +6433,7 @@
         <v/>
       </c>
       <c r="Z79" s="7">
-        <f>IF(OR(Y79="",'多次统计数据'!$B$8=""),"",Y79-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE79="",'多次统计数据'!$B$8=""),"",AE79-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA79" s="10">
@@ -6129,6 +6449,10 @@
         <v/>
       </c>
       <c r="AD79" s="2" t="n"/>
+      <c r="AE79" s="7">
+        <f>IF(OR(X79="",C79="",C79&lt;=0),"",X79/C79)</f>
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n"/>
@@ -6181,7 +6505,7 @@
         <v/>
       </c>
       <c r="Z80" s="7">
-        <f>IF(OR(Y80="",'多次统计数据'!$B$8=""),"",Y80-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE80="",'多次统计数据'!$B$8=""),"",AE80-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA80" s="10">
@@ -6197,6 +6521,10 @@
         <v/>
       </c>
       <c r="AD80" s="2" t="n"/>
+      <c r="AE80" s="7">
+        <f>IF(OR(X80="",C80="",C80&lt;=0),"",X80/C80)</f>
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n"/>
@@ -6249,7 +6577,7 @@
         <v/>
       </c>
       <c r="Z81" s="7">
-        <f>IF(OR(Y81="",'多次统计数据'!$B$8=""),"",Y81-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE81="",'多次统计数据'!$B$8=""),"",AE81-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA81" s="10">
@@ -6265,6 +6593,10 @@
         <v/>
       </c>
       <c r="AD81" s="2" t="n"/>
+      <c r="AE81" s="7">
+        <f>IF(OR(X81="",C81="",C81&lt;=0),"",X81/C81)</f>
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n"/>
@@ -6317,7 +6649,7 @@
         <v/>
       </c>
       <c r="Z82" s="7">
-        <f>IF(OR(Y82="",'多次统计数据'!$B$8=""),"",Y82-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE82="",'多次统计数据'!$B$8=""),"",AE82-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA82" s="10">
@@ -6333,6 +6665,10 @@
         <v/>
       </c>
       <c r="AD82" s="2" t="n"/>
+      <c r="AE82" s="7">
+        <f>IF(OR(X82="",C82="",C82&lt;=0),"",X82/C82)</f>
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n"/>
@@ -6385,7 +6721,7 @@
         <v/>
       </c>
       <c r="Z83" s="7">
-        <f>IF(OR(Y83="",'多次统计数据'!$B$8=""),"",Y83-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE83="",'多次统计数据'!$B$8=""),"",AE83-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA83" s="10">
@@ -6401,6 +6737,10 @@
         <v/>
       </c>
       <c r="AD83" s="2" t="n"/>
+      <c r="AE83" s="7">
+        <f>IF(OR(X83="",C83="",C83&lt;=0),"",X83/C83)</f>
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n"/>
@@ -6453,7 +6793,7 @@
         <v/>
       </c>
       <c r="Z84" s="7">
-        <f>IF(OR(Y84="",'多次统计数据'!$B$8=""),"",Y84-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE84="",'多次统计数据'!$B$8=""),"",AE84-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA84" s="10">
@@ -6469,6 +6809,10 @@
         <v/>
       </c>
       <c r="AD84" s="2" t="n"/>
+      <c r="AE84" s="7">
+        <f>IF(OR(X84="",C84="",C84&lt;=0),"",X84/C84)</f>
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n"/>
@@ -6521,7 +6865,7 @@
         <v/>
       </c>
       <c r="Z85" s="7">
-        <f>IF(OR(Y85="",'多次统计数据'!$B$8=""),"",Y85-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE85="",'多次统计数据'!$B$8=""),"",AE85-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA85" s="10">
@@ -6537,6 +6881,10 @@
         <v/>
       </c>
       <c r="AD85" s="2" t="n"/>
+      <c r="AE85" s="7">
+        <f>IF(OR(X85="",C85="",C85&lt;=0),"",X85/C85)</f>
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n"/>
@@ -6589,7 +6937,7 @@
         <v/>
       </c>
       <c r="Z86" s="7">
-        <f>IF(OR(Y86="",'多次统计数据'!$B$8=""),"",Y86-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE86="",'多次统计数据'!$B$8=""),"",AE86-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA86" s="10">
@@ -6605,6 +6953,10 @@
         <v/>
       </c>
       <c r="AD86" s="2" t="n"/>
+      <c r="AE86" s="7">
+        <f>IF(OR(X86="",C86="",C86&lt;=0),"",X86/C86)</f>
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n"/>
@@ -6657,7 +7009,7 @@
         <v/>
       </c>
       <c r="Z87" s="7">
-        <f>IF(OR(Y87="",'多次统计数据'!$B$8=""),"",Y87-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE87="",'多次统计数据'!$B$8=""),"",AE87-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA87" s="10">
@@ -6673,6 +7025,10 @@
         <v/>
       </c>
       <c r="AD87" s="2" t="n"/>
+      <c r="AE87" s="7">
+        <f>IF(OR(X87="",C87="",C87&lt;=0),"",X87/C87)</f>
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n"/>
@@ -6725,7 +7081,7 @@
         <v/>
       </c>
       <c r="Z88" s="7">
-        <f>IF(OR(Y88="",'多次统计数据'!$B$8=""),"",Y88-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE88="",'多次统计数据'!$B$8=""),"",AE88-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA88" s="10">
@@ -6741,6 +7097,10 @@
         <v/>
       </c>
       <c r="AD88" s="2" t="n"/>
+      <c r="AE88" s="7">
+        <f>IF(OR(X88="",C88="",C88&lt;=0),"",X88/C88)</f>
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n"/>
@@ -6793,7 +7153,7 @@
         <v/>
       </c>
       <c r="Z89" s="7">
-        <f>IF(OR(Y89="",'多次统计数据'!$B$8=""),"",Y89-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE89="",'多次统计数据'!$B$8=""),"",AE89-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA89" s="10">
@@ -6809,6 +7169,10 @@
         <v/>
       </c>
       <c r="AD89" s="2" t="n"/>
+      <c r="AE89" s="7">
+        <f>IF(OR(X89="",C89="",C89&lt;=0),"",X89/C89)</f>
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n"/>
@@ -6861,7 +7225,7 @@
         <v/>
       </c>
       <c r="Z90" s="7">
-        <f>IF(OR(Y90="",'多次统计数据'!$B$8=""),"",Y90-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE90="",'多次统计数据'!$B$8=""),"",AE90-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA90" s="10">
@@ -6877,6 +7241,10 @@
         <v/>
       </c>
       <c r="AD90" s="2" t="n"/>
+      <c r="AE90" s="7">
+        <f>IF(OR(X90="",C90="",C90&lt;=0),"",X90/C90)</f>
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n"/>
@@ -6929,7 +7297,7 @@
         <v/>
       </c>
       <c r="Z91" s="7">
-        <f>IF(OR(Y91="",'多次统计数据'!$B$8=""),"",Y91-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE91="",'多次统计数据'!$B$8=""),"",AE91-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA91" s="10">
@@ -6945,6 +7313,10 @@
         <v/>
       </c>
       <c r="AD91" s="2" t="n"/>
+      <c r="AE91" s="7">
+        <f>IF(OR(X91="",C91="",C91&lt;=0),"",X91/C91)</f>
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n"/>
@@ -6997,7 +7369,7 @@
         <v/>
       </c>
       <c r="Z92" s="7">
-        <f>IF(OR(Y92="",'多次统计数据'!$B$8=""),"",Y92-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE92="",'多次统计数据'!$B$8=""),"",AE92-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA92" s="10">
@@ -7013,6 +7385,10 @@
         <v/>
       </c>
       <c r="AD92" s="2" t="n"/>
+      <c r="AE92" s="7">
+        <f>IF(OR(X92="",C92="",C92&lt;=0),"",X92/C92)</f>
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n"/>
@@ -7065,7 +7441,7 @@
         <v/>
       </c>
       <c r="Z93" s="7">
-        <f>IF(OR(Y93="",'多次统计数据'!$B$8=""),"",Y93-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE93="",'多次统计数据'!$B$8=""),"",AE93-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA93" s="10">
@@ -7081,6 +7457,10 @@
         <v/>
       </c>
       <c r="AD93" s="2" t="n"/>
+      <c r="AE93" s="7">
+        <f>IF(OR(X93="",C93="",C93&lt;=0),"",X93/C93)</f>
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n"/>
@@ -7133,7 +7513,7 @@
         <v/>
       </c>
       <c r="Z94" s="7">
-        <f>IF(OR(Y94="",'多次统计数据'!$B$8=""),"",Y94-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE94="",'多次统计数据'!$B$8=""),"",AE94-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA94" s="10">
@@ -7149,6 +7529,10 @@
         <v/>
       </c>
       <c r="AD94" s="2" t="n"/>
+      <c r="AE94" s="7">
+        <f>IF(OR(X94="",C94="",C94&lt;=0),"",X94/C94)</f>
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n"/>
@@ -7201,7 +7585,7 @@
         <v/>
       </c>
       <c r="Z95" s="7">
-        <f>IF(OR(Y95="",'多次统计数据'!$B$8=""),"",Y95-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE95="",'多次统计数据'!$B$8=""),"",AE95-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA95" s="10">
@@ -7217,6 +7601,10 @@
         <v/>
       </c>
       <c r="AD95" s="2" t="n"/>
+      <c r="AE95" s="7">
+        <f>IF(OR(X95="",C95="",C95&lt;=0),"",X95/C95)</f>
+        <v/>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n"/>
@@ -7269,7 +7657,7 @@
         <v/>
       </c>
       <c r="Z96" s="7">
-        <f>IF(OR(Y96="",'多次统计数据'!$B$8=""),"",Y96-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE96="",'多次统计数据'!$B$8=""),"",AE96-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA96" s="10">
@@ -7285,6 +7673,10 @@
         <v/>
       </c>
       <c r="AD96" s="2" t="n"/>
+      <c r="AE96" s="7">
+        <f>IF(OR(X96="",C96="",C96&lt;=0),"",X96/C96)</f>
+        <v/>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n"/>
@@ -7337,7 +7729,7 @@
         <v/>
       </c>
       <c r="Z97" s="7">
-        <f>IF(OR(Y97="",'多次统计数据'!$B$8=""),"",Y97-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE97="",'多次统计数据'!$B$8=""),"",AE97-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA97" s="10">
@@ -7353,6 +7745,10 @@
         <v/>
       </c>
       <c r="AD97" s="2" t="n"/>
+      <c r="AE97" s="7">
+        <f>IF(OR(X97="",C97="",C97&lt;=0),"",X97/C97)</f>
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n"/>
@@ -7405,7 +7801,7 @@
         <v/>
       </c>
       <c r="Z98" s="7">
-        <f>IF(OR(Y98="",'多次统计数据'!$B$8=""),"",Y98-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE98="",'多次统计数据'!$B$8=""),"",AE98-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA98" s="10">
@@ -7421,6 +7817,10 @@
         <v/>
       </c>
       <c r="AD98" s="2" t="n"/>
+      <c r="AE98" s="7">
+        <f>IF(OR(X98="",C98="",C98&lt;=0),"",X98/C98)</f>
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n"/>
@@ -7473,7 +7873,7 @@
         <v/>
       </c>
       <c r="Z99" s="7">
-        <f>IF(OR(Y99="",'多次统计数据'!$B$8=""),"",Y99-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE99="",'多次统计数据'!$B$8=""),"",AE99-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA99" s="10">
@@ -7489,6 +7889,10 @@
         <v/>
       </c>
       <c r="AD99" s="2" t="n"/>
+      <c r="AE99" s="7">
+        <f>IF(OR(X99="",C99="",C99&lt;=0),"",X99/C99)</f>
+        <v/>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n"/>
@@ -7541,7 +7945,7 @@
         <v/>
       </c>
       <c r="Z100" s="7">
-        <f>IF(OR(Y100="",'多次统计数据'!$B$8=""),"",Y100-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE100="",'多次统计数据'!$B$8=""),"",AE100-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA100" s="10">
@@ -7557,6 +7961,10 @@
         <v/>
       </c>
       <c r="AD100" s="2" t="n"/>
+      <c r="AE100" s="7">
+        <f>IF(OR(X100="",C100="",C100&lt;=0),"",X100/C100)</f>
+        <v/>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n"/>
@@ -7609,7 +8017,7 @@
         <v/>
       </c>
       <c r="Z101" s="7">
-        <f>IF(OR(Y101="",'多次统计数据'!$B$8=""),"",Y101-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE101="",'多次统计数据'!$B$8=""),"",AE101-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA101" s="10">
@@ -7625,6 +8033,10 @@
         <v/>
       </c>
       <c r="AD101" s="2" t="n"/>
+      <c r="AE101" s="7">
+        <f>IF(OR(X101="",C101="",C101&lt;=0),"",X101/C101)</f>
+        <v/>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n"/>
@@ -7677,7 +8089,7 @@
         <v/>
       </c>
       <c r="Z102" s="7">
-        <f>IF(OR(Y102="",'多次统计数据'!$B$8=""),"",Y102-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE102="",'多次统计数据'!$B$8=""),"",AE102-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA102" s="10">
@@ -7693,6 +8105,10 @@
         <v/>
       </c>
       <c r="AD102" s="2" t="n"/>
+      <c r="AE102" s="7">
+        <f>IF(OR(X102="",C102="",C102&lt;=0),"",X102/C102)</f>
+        <v/>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n"/>
@@ -7745,7 +8161,7 @@
         <v/>
       </c>
       <c r="Z103" s="7">
-        <f>IF(OR(Y103="",'多次统计数据'!$B$8=""),"",Y103-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE103="",'多次统计数据'!$B$8=""),"",AE103-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA103" s="10">
@@ -7761,6 +8177,10 @@
         <v/>
       </c>
       <c r="AD103" s="2" t="n"/>
+      <c r="AE103" s="7">
+        <f>IF(OR(X103="",C103="",C103&lt;=0),"",X103/C103)</f>
+        <v/>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n"/>
@@ -7813,7 +8233,7 @@
         <v/>
       </c>
       <c r="Z104" s="7">
-        <f>IF(OR(Y104="",'多次统计数据'!$B$8=""),"",Y104-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE104="",'多次统计数据'!$B$8=""),"",AE104-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA104" s="10">
@@ -7829,6 +8249,10 @@
         <v/>
       </c>
       <c r="AD104" s="2" t="n"/>
+      <c r="AE104" s="7">
+        <f>IF(OR(X104="",C104="",C104&lt;=0),"",X104/C104)</f>
+        <v/>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n"/>
@@ -7881,7 +8305,7 @@
         <v/>
       </c>
       <c r="Z105" s="7">
-        <f>IF(OR(Y105="",'多次统计数据'!$B$8=""),"",Y105-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE105="",'多次统计数据'!$B$8=""),"",AE105-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA105" s="10">
@@ -7897,6 +8321,10 @@
         <v/>
       </c>
       <c r="AD105" s="2" t="n"/>
+      <c r="AE105" s="7">
+        <f>IF(OR(X105="",C105="",C105&lt;=0),"",X105/C105)</f>
+        <v/>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n"/>
@@ -7949,7 +8377,7 @@
         <v/>
       </c>
       <c r="Z106" s="7">
-        <f>IF(OR(Y106="",'多次统计数据'!$B$8=""),"",Y106-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE106="",'多次统计数据'!$B$8=""),"",AE106-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA106" s="10">
@@ -7965,6 +8393,10 @@
         <v/>
       </c>
       <c r="AD106" s="2" t="n"/>
+      <c r="AE106" s="7">
+        <f>IF(OR(X106="",C106="",C106&lt;=0),"",X106/C106)</f>
+        <v/>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n"/>
@@ -8017,7 +8449,7 @@
         <v/>
       </c>
       <c r="Z107" s="7">
-        <f>IF(OR(Y107="",'多次统计数据'!$B$8=""),"",Y107-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE107="",'多次统计数据'!$B$8=""),"",AE107-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA107" s="10">
@@ -8033,6 +8465,10 @@
         <v/>
       </c>
       <c r="AD107" s="2" t="n"/>
+      <c r="AE107" s="7">
+        <f>IF(OR(X107="",C107="",C107&lt;=0),"",X107/C107)</f>
+        <v/>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n"/>
@@ -8085,7 +8521,7 @@
         <v/>
       </c>
       <c r="Z108" s="7">
-        <f>IF(OR(Y108="",'多次统计数据'!$B$8=""),"",Y108-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE108="",'多次统计数据'!$B$8=""),"",AE108-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA108" s="10">
@@ -8101,6 +8537,10 @@
         <v/>
       </c>
       <c r="AD108" s="2" t="n"/>
+      <c r="AE108" s="7">
+        <f>IF(OR(X108="",C108="",C108&lt;=0),"",X108/C108)</f>
+        <v/>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n"/>
@@ -8153,7 +8593,7 @@
         <v/>
       </c>
       <c r="Z109" s="7">
-        <f>IF(OR(Y109="",'多次统计数据'!$B$8=""),"",Y109-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE109="",'多次统计数据'!$B$8=""),"",AE109-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA109" s="10">
@@ -8169,6 +8609,10 @@
         <v/>
       </c>
       <c r="AD109" s="2" t="n"/>
+      <c r="AE109" s="7">
+        <f>IF(OR(X109="",C109="",C109&lt;=0),"",X109/C109)</f>
+        <v/>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n"/>
@@ -8221,7 +8665,7 @@
         <v/>
       </c>
       <c r="Z110" s="7">
-        <f>IF(OR(Y110="",'多次统计数据'!$B$8=""),"",Y110-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE110="",'多次统计数据'!$B$8=""),"",AE110-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA110" s="10">
@@ -8237,6 +8681,10 @@
         <v/>
       </c>
       <c r="AD110" s="2" t="n"/>
+      <c r="AE110" s="7">
+        <f>IF(OR(X110="",C110="",C110&lt;=0),"",X110/C110)</f>
+        <v/>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n"/>
@@ -8289,7 +8737,7 @@
         <v/>
       </c>
       <c r="Z111" s="7">
-        <f>IF(OR(Y111="",'多次统计数据'!$B$8=""),"",Y111-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE111="",'多次统计数据'!$B$8=""),"",AE111-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA111" s="10">
@@ -8305,6 +8753,10 @@
         <v/>
       </c>
       <c r="AD111" s="2" t="n"/>
+      <c r="AE111" s="7">
+        <f>IF(OR(X111="",C111="",C111&lt;=0),"",X111/C111)</f>
+        <v/>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n"/>
@@ -8357,7 +8809,7 @@
         <v/>
       </c>
       <c r="Z112" s="7">
-        <f>IF(OR(Y112="",'多次统计数据'!$B$8=""),"",Y112-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE112="",'多次统计数据'!$B$8=""),"",AE112-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA112" s="10">
@@ -8373,6 +8825,10 @@
         <v/>
       </c>
       <c r="AD112" s="2" t="n"/>
+      <c r="AE112" s="7">
+        <f>IF(OR(X112="",C112="",C112&lt;=0),"",X112/C112)</f>
+        <v/>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n"/>
@@ -8425,7 +8881,7 @@
         <v/>
       </c>
       <c r="Z113" s="7">
-        <f>IF(OR(Y113="",'多次统计数据'!$B$8=""),"",Y113-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE113="",'多次统计数据'!$B$8=""),"",AE113-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA113" s="10">
@@ -8441,6 +8897,10 @@
         <v/>
       </c>
       <c r="AD113" s="2" t="n"/>
+      <c r="AE113" s="7">
+        <f>IF(OR(X113="",C113="",C113&lt;=0),"",X113/C113)</f>
+        <v/>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n"/>
@@ -8493,7 +8953,7 @@
         <v/>
       </c>
       <c r="Z114" s="7">
-        <f>IF(OR(Y114="",'多次统计数据'!$B$8=""),"",Y114-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE114="",'多次统计数据'!$B$8=""),"",AE114-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA114" s="10">
@@ -8509,6 +8969,10 @@
         <v/>
       </c>
       <c r="AD114" s="2" t="n"/>
+      <c r="AE114" s="7">
+        <f>IF(OR(X114="",C114="",C114&lt;=0),"",X114/C114)</f>
+        <v/>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n"/>
@@ -8561,7 +9025,7 @@
         <v/>
       </c>
       <c r="Z115" s="7">
-        <f>IF(OR(Y115="",'多次统计数据'!$B$8=""),"",Y115-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE115="",'多次统计数据'!$B$8=""),"",AE115-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA115" s="10">
@@ -8577,6 +9041,10 @@
         <v/>
       </c>
       <c r="AD115" s="2" t="n"/>
+      <c r="AE115" s="7">
+        <f>IF(OR(X115="",C115="",C115&lt;=0),"",X115/C115)</f>
+        <v/>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n"/>
@@ -8629,7 +9097,7 @@
         <v/>
       </c>
       <c r="Z116" s="7">
-        <f>IF(OR(Y116="",'多次统计数据'!$B$8=""),"",Y116-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE116="",'多次统计数据'!$B$8=""),"",AE116-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA116" s="10">
@@ -8645,6 +9113,10 @@
         <v/>
       </c>
       <c r="AD116" s="2" t="n"/>
+      <c r="AE116" s="7">
+        <f>IF(OR(X116="",C116="",C116&lt;=0),"",X116/C116)</f>
+        <v/>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n"/>
@@ -8697,7 +9169,7 @@
         <v/>
       </c>
       <c r="Z117" s="7">
-        <f>IF(OR(Y117="",'多次统计数据'!$B$8=""),"",Y117-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE117="",'多次统计数据'!$B$8=""),"",AE117-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA117" s="10">
@@ -8713,6 +9185,10 @@
         <v/>
       </c>
       <c r="AD117" s="2" t="n"/>
+      <c r="AE117" s="7">
+        <f>IF(OR(X117="",C117="",C117&lt;=0),"",X117/C117)</f>
+        <v/>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n"/>
@@ -8765,7 +9241,7 @@
         <v/>
       </c>
       <c r="Z118" s="7">
-        <f>IF(OR(Y118="",'多次统计数据'!$B$8=""),"",Y118-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE118="",'多次统计数据'!$B$8=""),"",AE118-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA118" s="10">
@@ -8781,6 +9257,10 @@
         <v/>
       </c>
       <c r="AD118" s="2" t="n"/>
+      <c r="AE118" s="7">
+        <f>IF(OR(X118="",C118="",C118&lt;=0),"",X118/C118)</f>
+        <v/>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n"/>
@@ -8833,7 +9313,7 @@
         <v/>
       </c>
       <c r="Z119" s="7">
-        <f>IF(OR(Y119="",'多次统计数据'!$B$8=""),"",Y119-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE119="",'多次统计数据'!$B$8=""),"",AE119-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA119" s="10">
@@ -8849,6 +9329,10 @@
         <v/>
       </c>
       <c r="AD119" s="2" t="n"/>
+      <c r="AE119" s="7">
+        <f>IF(OR(X119="",C119="",C119&lt;=0),"",X119/C119)</f>
+        <v/>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n"/>
@@ -8901,7 +9385,7 @@
         <v/>
       </c>
       <c r="Z120" s="7">
-        <f>IF(OR(Y120="",'多次统计数据'!$B$8=""),"",Y120-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE120="",'多次统计数据'!$B$8=""),"",AE120-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA120" s="10">
@@ -8917,6 +9401,10 @@
         <v/>
       </c>
       <c r="AD120" s="2" t="n"/>
+      <c r="AE120" s="7">
+        <f>IF(OR(X120="",C120="",C120&lt;=0),"",X120/C120)</f>
+        <v/>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n"/>
@@ -8969,7 +9457,7 @@
         <v/>
       </c>
       <c r="Z121" s="7">
-        <f>IF(OR(Y121="",'多次统计数据'!$B$8=""),"",Y121-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE121="",'多次统计数据'!$B$8=""),"",AE121-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA121" s="10">
@@ -8985,6 +9473,10 @@
         <v/>
       </c>
       <c r="AD121" s="2" t="n"/>
+      <c r="AE121" s="7">
+        <f>IF(OR(X121="",C121="",C121&lt;=0),"",X121/C121)</f>
+        <v/>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n"/>
@@ -9037,7 +9529,7 @@
         <v/>
       </c>
       <c r="Z122" s="7">
-        <f>IF(OR(Y122="",'多次统计数据'!$B$8=""),"",Y122-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE122="",'多次统计数据'!$B$8=""),"",AE122-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA122" s="10">
@@ -9053,6 +9545,10 @@
         <v/>
       </c>
       <c r="AD122" s="2" t="n"/>
+      <c r="AE122" s="7">
+        <f>IF(OR(X122="",C122="",C122&lt;=0),"",X122/C122)</f>
+        <v/>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n"/>
@@ -9105,7 +9601,7 @@
         <v/>
       </c>
       <c r="Z123" s="7">
-        <f>IF(OR(Y123="",'多次统计数据'!$B$8=""),"",Y123-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE123="",'多次统计数据'!$B$8=""),"",AE123-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA123" s="10">
@@ -9121,6 +9617,10 @@
         <v/>
       </c>
       <c r="AD123" s="2" t="n"/>
+      <c r="AE123" s="7">
+        <f>IF(OR(X123="",C123="",C123&lt;=0),"",X123/C123)</f>
+        <v/>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n"/>
@@ -9173,7 +9673,7 @@
         <v/>
       </c>
       <c r="Z124" s="7">
-        <f>IF(OR(Y124="",'多次统计数据'!$B$8=""),"",Y124-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE124="",'多次统计数据'!$B$8=""),"",AE124-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA124" s="10">
@@ -9189,6 +9689,10 @@
         <v/>
       </c>
       <c r="AD124" s="2" t="n"/>
+      <c r="AE124" s="7">
+        <f>IF(OR(X124="",C124="",C124&lt;=0),"",X124/C124)</f>
+        <v/>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n"/>
@@ -9241,7 +9745,7 @@
         <v/>
       </c>
       <c r="Z125" s="7">
-        <f>IF(OR(Y125="",'多次统计数据'!$B$8=""),"",Y125-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE125="",'多次统计数据'!$B$8=""),"",AE125-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA125" s="10">
@@ -9257,6 +9761,10 @@
         <v/>
       </c>
       <c r="AD125" s="2" t="n"/>
+      <c r="AE125" s="7">
+        <f>IF(OR(X125="",C125="",C125&lt;=0),"",X125/C125)</f>
+        <v/>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n"/>
@@ -9309,7 +9817,7 @@
         <v/>
       </c>
       <c r="Z126" s="7">
-        <f>IF(OR(Y126="",'多次统计数据'!$B$8=""),"",Y126-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE126="",'多次统计数据'!$B$8=""),"",AE126-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA126" s="10">
@@ -9325,6 +9833,10 @@
         <v/>
       </c>
       <c r="AD126" s="2" t="n"/>
+      <c r="AE126" s="7">
+        <f>IF(OR(X126="",C126="",C126&lt;=0),"",X126/C126)</f>
+        <v/>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n"/>
@@ -9377,7 +9889,7 @@
         <v/>
       </c>
       <c r="Z127" s="7">
-        <f>IF(OR(Y127="",'多次统计数据'!$B$8=""),"",Y127-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE127="",'多次统计数据'!$B$8=""),"",AE127-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA127" s="10">
@@ -9393,6 +9905,10 @@
         <v/>
       </c>
       <c r="AD127" s="2" t="n"/>
+      <c r="AE127" s="7">
+        <f>IF(OR(X127="",C127="",C127&lt;=0),"",X127/C127)</f>
+        <v/>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="n"/>
@@ -9445,7 +9961,7 @@
         <v/>
       </c>
       <c r="Z128" s="7">
-        <f>IF(OR(Y128="",'多次统计数据'!$B$8=""),"",Y128-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE128="",'多次统计数据'!$B$8=""),"",AE128-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA128" s="10">
@@ -9461,6 +9977,10 @@
         <v/>
       </c>
       <c r="AD128" s="2" t="n"/>
+      <c r="AE128" s="7">
+        <f>IF(OR(X128="",C128="",C128&lt;=0),"",X128/C128)</f>
+        <v/>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="n"/>
@@ -9513,7 +10033,7 @@
         <v/>
       </c>
       <c r="Z129" s="7">
-        <f>IF(OR(Y129="",'多次统计数据'!$B$8=""),"",Y129-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE129="",'多次统计数据'!$B$8=""),"",AE129-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA129" s="10">
@@ -9529,6 +10049,10 @@
         <v/>
       </c>
       <c r="AD129" s="2" t="n"/>
+      <c r="AE129" s="7">
+        <f>IF(OR(X129="",C129="",C129&lt;=0),"",X129/C129)</f>
+        <v/>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="n"/>
@@ -9581,7 +10105,7 @@
         <v/>
       </c>
       <c r="Z130" s="7">
-        <f>IF(OR(Y130="",'多次统计数据'!$B$8=""),"",Y130-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE130="",'多次统计数据'!$B$8=""),"",AE130-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA130" s="10">
@@ -9597,6 +10121,10 @@
         <v/>
       </c>
       <c r="AD130" s="2" t="n"/>
+      <c r="AE130" s="7">
+        <f>IF(OR(X130="",C130="",C130&lt;=0),"",X130/C130)</f>
+        <v/>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="n"/>
@@ -9649,7 +10177,7 @@
         <v/>
       </c>
       <c r="Z131" s="7">
-        <f>IF(OR(Y131="",'多次统计数据'!$B$8=""),"",Y131-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE131="",'多次统计数据'!$B$8=""),"",AE131-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA131" s="10">
@@ -9665,6 +10193,10 @@
         <v/>
       </c>
       <c r="AD131" s="2" t="n"/>
+      <c r="AE131" s="7">
+        <f>IF(OR(X131="",C131="",C131&lt;=0),"",X131/C131)</f>
+        <v/>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="n"/>
@@ -9717,7 +10249,7 @@
         <v/>
       </c>
       <c r="Z132" s="7">
-        <f>IF(OR(Y132="",'多次统计数据'!$B$8=""),"",Y132-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE132="",'多次统计数据'!$B$8=""),"",AE132-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA132" s="10">
@@ -9733,6 +10265,10 @@
         <v/>
       </c>
       <c r="AD132" s="2" t="n"/>
+      <c r="AE132" s="7">
+        <f>IF(OR(X132="",C132="",C132&lt;=0),"",X132/C132)</f>
+        <v/>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="n"/>
@@ -9785,7 +10321,7 @@
         <v/>
       </c>
       <c r="Z133" s="7">
-        <f>IF(OR(Y133="",'多次统计数据'!$B$8=""),"",Y133-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE133="",'多次统计数据'!$B$8=""),"",AE133-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA133" s="10">
@@ -9801,6 +10337,10 @@
         <v/>
       </c>
       <c r="AD133" s="2" t="n"/>
+      <c r="AE133" s="7">
+        <f>IF(OR(X133="",C133="",C133&lt;=0),"",X133/C133)</f>
+        <v/>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="n"/>
@@ -9853,7 +10393,7 @@
         <v/>
       </c>
       <c r="Z134" s="7">
-        <f>IF(OR(Y134="",'多次统计数据'!$B$8=""),"",Y134-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE134="",'多次统计数据'!$B$8=""),"",AE134-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA134" s="10">
@@ -9869,6 +10409,10 @@
         <v/>
       </c>
       <c r="AD134" s="2" t="n"/>
+      <c r="AE134" s="7">
+        <f>IF(OR(X134="",C134="",C134&lt;=0),"",X134/C134)</f>
+        <v/>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="n"/>
@@ -9921,7 +10465,7 @@
         <v/>
       </c>
       <c r="Z135" s="7">
-        <f>IF(OR(Y135="",'多次统计数据'!$B$8=""),"",Y135-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE135="",'多次统计数据'!$B$8=""),"",AE135-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA135" s="10">
@@ -9937,6 +10481,10 @@
         <v/>
       </c>
       <c r="AD135" s="2" t="n"/>
+      <c r="AE135" s="7">
+        <f>IF(OR(X135="",C135="",C135&lt;=0),"",X135/C135)</f>
+        <v/>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="n"/>
@@ -9989,7 +10537,7 @@
         <v/>
       </c>
       <c r="Z136" s="7">
-        <f>IF(OR(Y136="",'多次统计数据'!$B$8=""),"",Y136-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE136="",'多次统计数据'!$B$8=""),"",AE136-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA136" s="10">
@@ -10005,6 +10553,10 @@
         <v/>
       </c>
       <c r="AD136" s="2" t="n"/>
+      <c r="AE136" s="7">
+        <f>IF(OR(X136="",C136="",C136&lt;=0),"",X136/C136)</f>
+        <v/>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="n"/>
@@ -10057,7 +10609,7 @@
         <v/>
       </c>
       <c r="Z137" s="7">
-        <f>IF(OR(Y137="",'多次统计数据'!$B$8=""),"",Y137-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE137="",'多次统计数据'!$B$8=""),"",AE137-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA137" s="10">
@@ -10073,6 +10625,10 @@
         <v/>
       </c>
       <c r="AD137" s="2" t="n"/>
+      <c r="AE137" s="7">
+        <f>IF(OR(X137="",C137="",C137&lt;=0),"",X137/C137)</f>
+        <v/>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="n"/>
@@ -10125,7 +10681,7 @@
         <v/>
       </c>
       <c r="Z138" s="7">
-        <f>IF(OR(Y138="",'多次统计数据'!$B$8=""),"",Y138-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE138="",'多次统计数据'!$B$8=""),"",AE138-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA138" s="10">
@@ -10141,6 +10697,10 @@
         <v/>
       </c>
       <c r="AD138" s="2" t="n"/>
+      <c r="AE138" s="7">
+        <f>IF(OR(X138="",C138="",C138&lt;=0),"",X138/C138)</f>
+        <v/>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="n"/>
@@ -10193,7 +10753,7 @@
         <v/>
       </c>
       <c r="Z139" s="7">
-        <f>IF(OR(Y139="",'多次统计数据'!$B$8=""),"",Y139-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE139="",'多次统计数据'!$B$8=""),"",AE139-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA139" s="10">
@@ -10209,6 +10769,10 @@
         <v/>
       </c>
       <c r="AD139" s="2" t="n"/>
+      <c r="AE139" s="7">
+        <f>IF(OR(X139="",C139="",C139&lt;=0),"",X139/C139)</f>
+        <v/>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="n"/>
@@ -10261,7 +10825,7 @@
         <v/>
       </c>
       <c r="Z140" s="7">
-        <f>IF(OR(Y140="",'多次统计数据'!$B$8=""),"",Y140-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE140="",'多次统计数据'!$B$8=""),"",AE140-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA140" s="10">
@@ -10277,6 +10841,10 @@
         <v/>
       </c>
       <c r="AD140" s="2" t="n"/>
+      <c r="AE140" s="7">
+        <f>IF(OR(X140="",C140="",C140&lt;=0),"",X140/C140)</f>
+        <v/>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="n"/>
@@ -10329,7 +10897,7 @@
         <v/>
       </c>
       <c r="Z141" s="7">
-        <f>IF(OR(Y141="",'多次统计数据'!$B$8=""),"",Y141-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE141="",'多次统计数据'!$B$8=""),"",AE141-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA141" s="10">
@@ -10345,6 +10913,10 @@
         <v/>
       </c>
       <c r="AD141" s="2" t="n"/>
+      <c r="AE141" s="7">
+        <f>IF(OR(X141="",C141="",C141&lt;=0),"",X141/C141)</f>
+        <v/>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="n"/>
@@ -10397,7 +10969,7 @@
         <v/>
       </c>
       <c r="Z142" s="7">
-        <f>IF(OR(Y142="",'多次统计数据'!$B$8=""),"",Y142-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE142="",'多次统计数据'!$B$8=""),"",AE142-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA142" s="10">
@@ -10413,6 +10985,10 @@
         <v/>
       </c>
       <c r="AD142" s="2" t="n"/>
+      <c r="AE142" s="7">
+        <f>IF(OR(X142="",C142="",C142&lt;=0),"",X142/C142)</f>
+        <v/>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="n"/>
@@ -10465,7 +11041,7 @@
         <v/>
       </c>
       <c r="Z143" s="7">
-        <f>IF(OR(Y143="",'多次统计数据'!$B$8=""),"",Y143-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE143="",'多次统计数据'!$B$8=""),"",AE143-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA143" s="10">
@@ -10481,6 +11057,10 @@
         <v/>
       </c>
       <c r="AD143" s="2" t="n"/>
+      <c r="AE143" s="7">
+        <f>IF(OR(X143="",C143="",C143&lt;=0),"",X143/C143)</f>
+        <v/>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="n"/>
@@ -10533,7 +11113,7 @@
         <v/>
       </c>
       <c r="Z144" s="7">
-        <f>IF(OR(Y144="",'多次统计数据'!$B$8=""),"",Y144-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE144="",'多次统计数据'!$B$8=""),"",AE144-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA144" s="10">
@@ -10549,6 +11129,10 @@
         <v/>
       </c>
       <c r="AD144" s="2" t="n"/>
+      <c r="AE144" s="7">
+        <f>IF(OR(X144="",C144="",C144&lt;=0),"",X144/C144)</f>
+        <v/>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="n"/>
@@ -10601,7 +11185,7 @@
         <v/>
       </c>
       <c r="Z145" s="7">
-        <f>IF(OR(Y145="",'多次统计数据'!$B$8=""),"",Y145-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE145="",'多次统计数据'!$B$8=""),"",AE145-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA145" s="10">
@@ -10617,6 +11201,10 @@
         <v/>
       </c>
       <c r="AD145" s="2" t="n"/>
+      <c r="AE145" s="7">
+        <f>IF(OR(X145="",C145="",C145&lt;=0),"",X145/C145)</f>
+        <v/>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="n"/>
@@ -10669,7 +11257,7 @@
         <v/>
       </c>
       <c r="Z146" s="7">
-        <f>IF(OR(Y146="",'多次统计数据'!$B$8=""),"",Y146-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE146="",'多次统计数据'!$B$8=""),"",AE146-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA146" s="10">
@@ -10685,6 +11273,10 @@
         <v/>
       </c>
       <c r="AD146" s="2" t="n"/>
+      <c r="AE146" s="7">
+        <f>IF(OR(X146="",C146="",C146&lt;=0),"",X146/C146)</f>
+        <v/>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="n"/>
@@ -10737,7 +11329,7 @@
         <v/>
       </c>
       <c r="Z147" s="7">
-        <f>IF(OR(Y147="",'多次统计数据'!$B$8=""),"",Y147-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE147="",'多次统计数据'!$B$8=""),"",AE147-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA147" s="10">
@@ -10753,6 +11345,10 @@
         <v/>
       </c>
       <c r="AD147" s="2" t="n"/>
+      <c r="AE147" s="7">
+        <f>IF(OR(X147="",C147="",C147&lt;=0),"",X147/C147)</f>
+        <v/>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="n"/>
@@ -10805,7 +11401,7 @@
         <v/>
       </c>
       <c r="Z148" s="7">
-        <f>IF(OR(Y148="",'多次统计数据'!$B$8=""),"",Y148-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE148="",'多次统计数据'!$B$8=""),"",AE148-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA148" s="10">
@@ -10821,6 +11417,10 @@
         <v/>
       </c>
       <c r="AD148" s="2" t="n"/>
+      <c r="AE148" s="7">
+        <f>IF(OR(X148="",C148="",C148&lt;=0),"",X148/C148)</f>
+        <v/>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="n"/>
@@ -10873,7 +11473,7 @@
         <v/>
       </c>
       <c r="Z149" s="7">
-        <f>IF(OR(Y149="",'多次统计数据'!$B$8=""),"",Y149-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE149="",'多次统计数据'!$B$8=""),"",AE149-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA149" s="10">
@@ -10889,6 +11489,10 @@
         <v/>
       </c>
       <c r="AD149" s="2" t="n"/>
+      <c r="AE149" s="7">
+        <f>IF(OR(X149="",C149="",C149&lt;=0),"",X149/C149)</f>
+        <v/>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="n"/>
@@ -10941,7 +11545,7 @@
         <v/>
       </c>
       <c r="Z150" s="7">
-        <f>IF(OR(Y150="",'多次统计数据'!$B$8=""),"",Y150-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE150="",'多次统计数据'!$B$8=""),"",AE150-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA150" s="10">
@@ -10957,6 +11561,10 @@
         <v/>
       </c>
       <c r="AD150" s="2" t="n"/>
+      <c r="AE150" s="7">
+        <f>IF(OR(X150="",C150="",C150&lt;=0),"",X150/C150)</f>
+        <v/>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="n"/>
@@ -11009,7 +11617,7 @@
         <v/>
       </c>
       <c r="Z151" s="7">
-        <f>IF(OR(Y151="",'多次统计数据'!$B$8=""),"",Y151-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE151="",'多次统计数据'!$B$8=""),"",AE151-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA151" s="10">
@@ -11025,6 +11633,10 @@
         <v/>
       </c>
       <c r="AD151" s="2" t="n"/>
+      <c r="AE151" s="7">
+        <f>IF(OR(X151="",C151="",C151&lt;=0),"",X151/C151)</f>
+        <v/>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="n"/>
@@ -11077,7 +11689,7 @@
         <v/>
       </c>
       <c r="Z152" s="7">
-        <f>IF(OR(Y152="",'多次统计数据'!$B$8=""),"",Y152-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE152="",'多次统计数据'!$B$8=""),"",AE152-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA152" s="10">
@@ -11093,6 +11705,10 @@
         <v/>
       </c>
       <c r="AD152" s="2" t="n"/>
+      <c r="AE152" s="7">
+        <f>IF(OR(X152="",C152="",C152&lt;=0),"",X152/C152)</f>
+        <v/>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="n"/>
@@ -11145,7 +11761,7 @@
         <v/>
       </c>
       <c r="Z153" s="7">
-        <f>IF(OR(Y153="",'多次统计数据'!$B$8=""),"",Y153-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE153="",'多次统计数据'!$B$8=""),"",AE153-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA153" s="10">
@@ -11161,6 +11777,10 @@
         <v/>
       </c>
       <c r="AD153" s="2" t="n"/>
+      <c r="AE153" s="7">
+        <f>IF(OR(X153="",C153="",C153&lt;=0),"",X153/C153)</f>
+        <v/>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="n"/>
@@ -11213,7 +11833,7 @@
         <v/>
       </c>
       <c r="Z154" s="7">
-        <f>IF(OR(Y154="",'多次统计数据'!$B$8=""),"",Y154-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE154="",'多次统计数据'!$B$8=""),"",AE154-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA154" s="10">
@@ -11229,6 +11849,10 @@
         <v/>
       </c>
       <c r="AD154" s="2" t="n"/>
+      <c r="AE154" s="7">
+        <f>IF(OR(X154="",C154="",C154&lt;=0),"",X154/C154)</f>
+        <v/>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="n"/>
@@ -11281,7 +11905,7 @@
         <v/>
       </c>
       <c r="Z155" s="7">
-        <f>IF(OR(Y155="",'多次统计数据'!$B$8=""),"",Y155-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE155="",'多次统计数据'!$B$8=""),"",AE155-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA155" s="10">
@@ -11297,6 +11921,10 @@
         <v/>
       </c>
       <c r="AD155" s="2" t="n"/>
+      <c r="AE155" s="7">
+        <f>IF(OR(X155="",C155="",C155&lt;=0),"",X155/C155)</f>
+        <v/>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="n"/>
@@ -11349,7 +11977,7 @@
         <v/>
       </c>
       <c r="Z156" s="7">
-        <f>IF(OR(Y156="",'多次统计数据'!$B$8=""),"",Y156-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE156="",'多次统计数据'!$B$8=""),"",AE156-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA156" s="10">
@@ -11365,6 +11993,10 @@
         <v/>
       </c>
       <c r="AD156" s="2" t="n"/>
+      <c r="AE156" s="7">
+        <f>IF(OR(X156="",C156="",C156&lt;=0),"",X156/C156)</f>
+        <v/>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="n"/>
@@ -11417,7 +12049,7 @@
         <v/>
       </c>
       <c r="Z157" s="7">
-        <f>IF(OR(Y157="",'多次统计数据'!$B$8=""),"",Y157-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE157="",'多次统计数据'!$B$8=""),"",AE157-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA157" s="10">
@@ -11433,6 +12065,10 @@
         <v/>
       </c>
       <c r="AD157" s="2" t="n"/>
+      <c r="AE157" s="7">
+        <f>IF(OR(X157="",C157="",C157&lt;=0),"",X157/C157)</f>
+        <v/>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="n"/>
@@ -11485,7 +12121,7 @@
         <v/>
       </c>
       <c r="Z158" s="7">
-        <f>IF(OR(Y158="",'多次统计数据'!$B$8=""),"",Y158-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE158="",'多次统计数据'!$B$8=""),"",AE158-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA158" s="10">
@@ -11501,6 +12137,10 @@
         <v/>
       </c>
       <c r="AD158" s="2" t="n"/>
+      <c r="AE158" s="7">
+        <f>IF(OR(X158="",C158="",C158&lt;=0),"",X158/C158)</f>
+        <v/>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="n"/>
@@ -11553,7 +12193,7 @@
         <v/>
       </c>
       <c r="Z159" s="7">
-        <f>IF(OR(Y159="",'多次统计数据'!$B$8=""),"",Y159-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE159="",'多次统计数据'!$B$8=""),"",AE159-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA159" s="10">
@@ -11569,6 +12209,10 @@
         <v/>
       </c>
       <c r="AD159" s="2" t="n"/>
+      <c r="AE159" s="7">
+        <f>IF(OR(X159="",C159="",C159&lt;=0),"",X159/C159)</f>
+        <v/>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="n"/>
@@ -11621,7 +12265,7 @@
         <v/>
       </c>
       <c r="Z160" s="7">
-        <f>IF(OR(Y160="",'多次统计数据'!$B$8=""),"",Y160-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE160="",'多次统计数据'!$B$8=""),"",AE160-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA160" s="10">
@@ -11637,6 +12281,10 @@
         <v/>
       </c>
       <c r="AD160" s="2" t="n"/>
+      <c r="AE160" s="7">
+        <f>IF(OR(X160="",C160="",C160&lt;=0),"",X160/C160)</f>
+        <v/>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="n"/>
@@ -11689,7 +12337,7 @@
         <v/>
       </c>
       <c r="Z161" s="7">
-        <f>IF(OR(Y161="",'多次统计数据'!$B$8=""),"",Y161-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE161="",'多次统计数据'!$B$8=""),"",AE161-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA161" s="10">
@@ -11705,6 +12353,10 @@
         <v/>
       </c>
       <c r="AD161" s="2" t="n"/>
+      <c r="AE161" s="7">
+        <f>IF(OR(X161="",C161="",C161&lt;=0),"",X161/C161)</f>
+        <v/>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="n"/>
@@ -11757,7 +12409,7 @@
         <v/>
       </c>
       <c r="Z162" s="7">
-        <f>IF(OR(Y162="",'多次统计数据'!$B$8=""),"",Y162-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE162="",'多次统计数据'!$B$8=""),"",AE162-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA162" s="10">
@@ -11773,6 +12425,10 @@
         <v/>
       </c>
       <c r="AD162" s="2" t="n"/>
+      <c r="AE162" s="7">
+        <f>IF(OR(X162="",C162="",C162&lt;=0),"",X162/C162)</f>
+        <v/>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="n"/>
@@ -11825,7 +12481,7 @@
         <v/>
       </c>
       <c r="Z163" s="7">
-        <f>IF(OR(Y163="",'多次统计数据'!$B$8=""),"",Y163-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE163="",'多次统计数据'!$B$8=""),"",AE163-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA163" s="10">
@@ -11841,6 +12497,10 @@
         <v/>
       </c>
       <c r="AD163" s="2" t="n"/>
+      <c r="AE163" s="7">
+        <f>IF(OR(X163="",C163="",C163&lt;=0),"",X163/C163)</f>
+        <v/>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="n"/>
@@ -11893,7 +12553,7 @@
         <v/>
       </c>
       <c r="Z164" s="7">
-        <f>IF(OR(Y164="",'多次统计数据'!$B$8=""),"",Y164-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE164="",'多次统计数据'!$B$8=""),"",AE164-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA164" s="10">
@@ -11909,6 +12569,10 @@
         <v/>
       </c>
       <c r="AD164" s="2" t="n"/>
+      <c r="AE164" s="7">
+        <f>IF(OR(X164="",C164="",C164&lt;=0),"",X164/C164)</f>
+        <v/>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="n"/>
@@ -11961,7 +12625,7 @@
         <v/>
       </c>
       <c r="Z165" s="7">
-        <f>IF(OR(Y165="",'多次统计数据'!$B$8=""),"",Y165-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE165="",'多次统计数据'!$B$8=""),"",AE165-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA165" s="10">
@@ -11977,6 +12641,10 @@
         <v/>
       </c>
       <c r="AD165" s="2" t="n"/>
+      <c r="AE165" s="7">
+        <f>IF(OR(X165="",C165="",C165&lt;=0),"",X165/C165)</f>
+        <v/>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="n"/>
@@ -12029,7 +12697,7 @@
         <v/>
       </c>
       <c r="Z166" s="7">
-        <f>IF(OR(Y166="",'多次统计数据'!$B$8=""),"",Y166-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE166="",'多次统计数据'!$B$8=""),"",AE166-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA166" s="10">
@@ -12045,6 +12713,10 @@
         <v/>
       </c>
       <c r="AD166" s="2" t="n"/>
+      <c r="AE166" s="7">
+        <f>IF(OR(X166="",C166="",C166&lt;=0),"",X166/C166)</f>
+        <v/>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="n"/>
@@ -12097,7 +12769,7 @@
         <v/>
       </c>
       <c r="Z167" s="7">
-        <f>IF(OR(Y167="",'多次统计数据'!$B$8=""),"",Y167-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE167="",'多次统计数据'!$B$8=""),"",AE167-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA167" s="10">
@@ -12113,6 +12785,10 @@
         <v/>
       </c>
       <c r="AD167" s="2" t="n"/>
+      <c r="AE167" s="7">
+        <f>IF(OR(X167="",C167="",C167&lt;=0),"",X167/C167)</f>
+        <v/>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="n"/>
@@ -12165,7 +12841,7 @@
         <v/>
       </c>
       <c r="Z168" s="7">
-        <f>IF(OR(Y168="",'多次统计数据'!$B$8=""),"",Y168-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE168="",'多次统计数据'!$B$8=""),"",AE168-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA168" s="10">
@@ -12181,6 +12857,10 @@
         <v/>
       </c>
       <c r="AD168" s="2" t="n"/>
+      <c r="AE168" s="7">
+        <f>IF(OR(X168="",C168="",C168&lt;=0),"",X168/C168)</f>
+        <v/>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="n"/>
@@ -12233,7 +12913,7 @@
         <v/>
       </c>
       <c r="Z169" s="7">
-        <f>IF(OR(Y169="",'多次统计数据'!$B$8=""),"",Y169-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE169="",'多次统计数据'!$B$8=""),"",AE169-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA169" s="10">
@@ -12249,6 +12929,10 @@
         <v/>
       </c>
       <c r="AD169" s="2" t="n"/>
+      <c r="AE169" s="7">
+        <f>IF(OR(X169="",C169="",C169&lt;=0),"",X169/C169)</f>
+        <v/>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="n"/>
@@ -12301,7 +12985,7 @@
         <v/>
       </c>
       <c r="Z170" s="7">
-        <f>IF(OR(Y170="",'多次统计数据'!$B$8=""),"",Y170-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE170="",'多次统计数据'!$B$8=""),"",AE170-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA170" s="10">
@@ -12317,6 +13001,10 @@
         <v/>
       </c>
       <c r="AD170" s="2" t="n"/>
+      <c r="AE170" s="7">
+        <f>IF(OR(X170="",C170="",C170&lt;=0),"",X170/C170)</f>
+        <v/>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="n"/>
@@ -12369,7 +13057,7 @@
         <v/>
       </c>
       <c r="Z171" s="7">
-        <f>IF(OR(Y171="",'多次统计数据'!$B$8=""),"",Y171-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE171="",'多次统计数据'!$B$8=""),"",AE171-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA171" s="10">
@@ -12385,6 +13073,10 @@
         <v/>
       </c>
       <c r="AD171" s="2" t="n"/>
+      <c r="AE171" s="7">
+        <f>IF(OR(X171="",C171="",C171&lt;=0),"",X171/C171)</f>
+        <v/>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="n"/>
@@ -12437,7 +13129,7 @@
         <v/>
       </c>
       <c r="Z172" s="7">
-        <f>IF(OR(Y172="",'多次统计数据'!$B$8=""),"",Y172-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE172="",'多次统计数据'!$B$8=""),"",AE172-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA172" s="10">
@@ -12453,6 +13145,10 @@
         <v/>
       </c>
       <c r="AD172" s="2" t="n"/>
+      <c r="AE172" s="7">
+        <f>IF(OR(X172="",C172="",C172&lt;=0),"",X172/C172)</f>
+        <v/>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="n"/>
@@ -12505,7 +13201,7 @@
         <v/>
       </c>
       <c r="Z173" s="7">
-        <f>IF(OR(Y173="",'多次统计数据'!$B$8=""),"",Y173-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE173="",'多次统计数据'!$B$8=""),"",AE173-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA173" s="10">
@@ -12521,6 +13217,10 @@
         <v/>
       </c>
       <c r="AD173" s="2" t="n"/>
+      <c r="AE173" s="7">
+        <f>IF(OR(X173="",C173="",C173&lt;=0),"",X173/C173)</f>
+        <v/>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="n"/>
@@ -12573,7 +13273,7 @@
         <v/>
       </c>
       <c r="Z174" s="7">
-        <f>IF(OR(Y174="",'多次统计数据'!$B$8=""),"",Y174-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE174="",'多次统计数据'!$B$8=""),"",AE174-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA174" s="10">
@@ -12589,6 +13289,10 @@
         <v/>
       </c>
       <c r="AD174" s="2" t="n"/>
+      <c r="AE174" s="7">
+        <f>IF(OR(X174="",C174="",C174&lt;=0),"",X174/C174)</f>
+        <v/>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="n"/>
@@ -12641,7 +13345,7 @@
         <v/>
       </c>
       <c r="Z175" s="7">
-        <f>IF(OR(Y175="",'多次统计数据'!$B$8=""),"",Y175-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE175="",'多次统计数据'!$B$8=""),"",AE175-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA175" s="10">
@@ -12657,6 +13361,10 @@
         <v/>
       </c>
       <c r="AD175" s="2" t="n"/>
+      <c r="AE175" s="7">
+        <f>IF(OR(X175="",C175="",C175&lt;=0),"",X175/C175)</f>
+        <v/>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="n"/>
@@ -12709,7 +13417,7 @@
         <v/>
       </c>
       <c r="Z176" s="7">
-        <f>IF(OR(Y176="",'多次统计数据'!$B$8=""),"",Y176-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE176="",'多次统计数据'!$B$8=""),"",AE176-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA176" s="10">
@@ -12725,6 +13433,10 @@
         <v/>
       </c>
       <c r="AD176" s="2" t="n"/>
+      <c r="AE176" s="7">
+        <f>IF(OR(X176="",C176="",C176&lt;=0),"",X176/C176)</f>
+        <v/>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="n"/>
@@ -12777,7 +13489,7 @@
         <v/>
       </c>
       <c r="Z177" s="7">
-        <f>IF(OR(Y177="",'多次统计数据'!$B$8=""),"",Y177-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE177="",'多次统计数据'!$B$8=""),"",AE177-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA177" s="10">
@@ -12793,6 +13505,10 @@
         <v/>
       </c>
       <c r="AD177" s="2" t="n"/>
+      <c r="AE177" s="7">
+        <f>IF(OR(X177="",C177="",C177&lt;=0),"",X177/C177)</f>
+        <v/>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="n"/>
@@ -12845,7 +13561,7 @@
         <v/>
       </c>
       <c r="Z178" s="7">
-        <f>IF(OR(Y178="",'多次统计数据'!$B$8=""),"",Y178-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE178="",'多次统计数据'!$B$8=""),"",AE178-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA178" s="10">
@@ -12861,6 +13577,10 @@
         <v/>
       </c>
       <c r="AD178" s="2" t="n"/>
+      <c r="AE178" s="7">
+        <f>IF(OR(X178="",C178="",C178&lt;=0),"",X178/C178)</f>
+        <v/>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="n"/>
@@ -12913,7 +13633,7 @@
         <v/>
       </c>
       <c r="Z179" s="7">
-        <f>IF(OR(Y179="",'多次统计数据'!$B$8=""),"",Y179-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE179="",'多次统计数据'!$B$8=""),"",AE179-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA179" s="10">
@@ -12929,6 +13649,10 @@
         <v/>
       </c>
       <c r="AD179" s="2" t="n"/>
+      <c r="AE179" s="7">
+        <f>IF(OR(X179="",C179="",C179&lt;=0),"",X179/C179)</f>
+        <v/>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="n"/>
@@ -12981,7 +13705,7 @@
         <v/>
       </c>
       <c r="Z180" s="7">
-        <f>IF(OR(Y180="",'多次统计数据'!$B$8=""),"",Y180-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE180="",'多次统计数据'!$B$8=""),"",AE180-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA180" s="10">
@@ -12997,6 +13721,10 @@
         <v/>
       </c>
       <c r="AD180" s="2" t="n"/>
+      <c r="AE180" s="7">
+        <f>IF(OR(X180="",C180="",C180&lt;=0),"",X180/C180)</f>
+        <v/>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="n"/>
@@ -13049,7 +13777,7 @@
         <v/>
       </c>
       <c r="Z181" s="7">
-        <f>IF(OR(Y181="",'多次统计数据'!$B$8=""),"",Y181-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE181="",'多次统计数据'!$B$8=""),"",AE181-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA181" s="10">
@@ -13065,6 +13793,10 @@
         <v/>
       </c>
       <c r="AD181" s="2" t="n"/>
+      <c r="AE181" s="7">
+        <f>IF(OR(X181="",C181="",C181&lt;=0),"",X181/C181)</f>
+        <v/>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="n"/>
@@ -13117,7 +13849,7 @@
         <v/>
       </c>
       <c r="Z182" s="7">
-        <f>IF(OR(Y182="",'多次统计数据'!$B$8=""),"",Y182-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE182="",'多次统计数据'!$B$8=""),"",AE182-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA182" s="10">
@@ -13133,6 +13865,10 @@
         <v/>
       </c>
       <c r="AD182" s="2" t="n"/>
+      <c r="AE182" s="7">
+        <f>IF(OR(X182="",C182="",C182&lt;=0),"",X182/C182)</f>
+        <v/>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="n"/>
@@ -13185,7 +13921,7 @@
         <v/>
       </c>
       <c r="Z183" s="7">
-        <f>IF(OR(Y183="",'多次统计数据'!$B$8=""),"",Y183-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE183="",'多次统计数据'!$B$8=""),"",AE183-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA183" s="10">
@@ -13201,6 +13937,10 @@
         <v/>
       </c>
       <c r="AD183" s="2" t="n"/>
+      <c r="AE183" s="7">
+        <f>IF(OR(X183="",C183="",C183&lt;=0),"",X183/C183)</f>
+        <v/>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="n"/>
@@ -13253,7 +13993,7 @@
         <v/>
       </c>
       <c r="Z184" s="7">
-        <f>IF(OR(Y184="",'多次统计数据'!$B$8=""),"",Y184-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE184="",'多次统计数据'!$B$8=""),"",AE184-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA184" s="10">
@@ -13269,6 +14009,10 @@
         <v/>
       </c>
       <c r="AD184" s="2" t="n"/>
+      <c r="AE184" s="7">
+        <f>IF(OR(X184="",C184="",C184&lt;=0),"",X184/C184)</f>
+        <v/>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="n"/>
@@ -13321,7 +14065,7 @@
         <v/>
       </c>
       <c r="Z185" s="7">
-        <f>IF(OR(Y185="",'多次统计数据'!$B$8=""),"",Y185-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE185="",'多次统计数据'!$B$8=""),"",AE185-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA185" s="10">
@@ -13337,6 +14081,10 @@
         <v/>
       </c>
       <c r="AD185" s="2" t="n"/>
+      <c r="AE185" s="7">
+        <f>IF(OR(X185="",C185="",C185&lt;=0),"",X185/C185)</f>
+        <v/>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="n"/>
@@ -13389,7 +14137,7 @@
         <v/>
       </c>
       <c r="Z186" s="7">
-        <f>IF(OR(Y186="",'多次统计数据'!$B$8=""),"",Y186-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE186="",'多次统计数据'!$B$8=""),"",AE186-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA186" s="10">
@@ -13405,6 +14153,10 @@
         <v/>
       </c>
       <c r="AD186" s="2" t="n"/>
+      <c r="AE186" s="7">
+        <f>IF(OR(X186="",C186="",C186&lt;=0),"",X186/C186)</f>
+        <v/>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="n"/>
@@ -13457,7 +14209,7 @@
         <v/>
       </c>
       <c r="Z187" s="7">
-        <f>IF(OR(Y187="",'多次统计数据'!$B$8=""),"",Y187-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE187="",'多次统计数据'!$B$8=""),"",AE187-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA187" s="10">
@@ -13473,6 +14225,10 @@
         <v/>
       </c>
       <c r="AD187" s="2" t="n"/>
+      <c r="AE187" s="7">
+        <f>IF(OR(X187="",C187="",C187&lt;=0),"",X187/C187)</f>
+        <v/>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="n"/>
@@ -13525,7 +14281,7 @@
         <v/>
       </c>
       <c r="Z188" s="7">
-        <f>IF(OR(Y188="",'多次统计数据'!$B$8=""),"",Y188-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE188="",'多次统计数据'!$B$8=""),"",AE188-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA188" s="10">
@@ -13541,6 +14297,10 @@
         <v/>
       </c>
       <c r="AD188" s="2" t="n"/>
+      <c r="AE188" s="7">
+        <f>IF(OR(X188="",C188="",C188&lt;=0),"",X188/C188)</f>
+        <v/>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="n"/>
@@ -13593,7 +14353,7 @@
         <v/>
       </c>
       <c r="Z189" s="7">
-        <f>IF(OR(Y189="",'多次统计数据'!$B$8=""),"",Y189-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE189="",'多次统计数据'!$B$8=""),"",AE189-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA189" s="10">
@@ -13609,6 +14369,10 @@
         <v/>
       </c>
       <c r="AD189" s="2" t="n"/>
+      <c r="AE189" s="7">
+        <f>IF(OR(X189="",C189="",C189&lt;=0),"",X189/C189)</f>
+        <v/>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="n"/>
@@ -13661,7 +14425,7 @@
         <v/>
       </c>
       <c r="Z190" s="7">
-        <f>IF(OR(Y190="",'多次统计数据'!$B$8=""),"",Y190-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE190="",'多次统计数据'!$B$8=""),"",AE190-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA190" s="10">
@@ -13677,6 +14441,10 @@
         <v/>
       </c>
       <c r="AD190" s="2" t="n"/>
+      <c r="AE190" s="7">
+        <f>IF(OR(X190="",C190="",C190&lt;=0),"",X190/C190)</f>
+        <v/>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="n"/>
@@ -13729,7 +14497,7 @@
         <v/>
       </c>
       <c r="Z191" s="7">
-        <f>IF(OR(Y191="",'多次统计数据'!$B$8=""),"",Y191-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE191="",'多次统计数据'!$B$8=""),"",AE191-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA191" s="10">
@@ -13745,6 +14513,10 @@
         <v/>
       </c>
       <c r="AD191" s="2" t="n"/>
+      <c r="AE191" s="7">
+        <f>IF(OR(X191="",C191="",C191&lt;=0),"",X191/C191)</f>
+        <v/>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="n"/>
@@ -13797,7 +14569,7 @@
         <v/>
       </c>
       <c r="Z192" s="7">
-        <f>IF(OR(Y192="",'多次统计数据'!$B$8=""),"",Y192-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE192="",'多次统计数据'!$B$8=""),"",AE192-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA192" s="10">
@@ -13813,6 +14585,10 @@
         <v/>
       </c>
       <c r="AD192" s="2" t="n"/>
+      <c r="AE192" s="7">
+        <f>IF(OR(X192="",C192="",C192&lt;=0),"",X192/C192)</f>
+        <v/>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="n"/>
@@ -13865,7 +14641,7 @@
         <v/>
       </c>
       <c r="Z193" s="7">
-        <f>IF(OR(Y193="",'多次统计数据'!$B$8=""),"",Y193-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE193="",'多次统计数据'!$B$8=""),"",AE193-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA193" s="10">
@@ -13881,6 +14657,10 @@
         <v/>
       </c>
       <c r="AD193" s="2" t="n"/>
+      <c r="AE193" s="7">
+        <f>IF(OR(X193="",C193="",C193&lt;=0),"",X193/C193)</f>
+        <v/>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="n"/>
@@ -13933,7 +14713,7 @@
         <v/>
       </c>
       <c r="Z194" s="7">
-        <f>IF(OR(Y194="",'多次统计数据'!$B$8=""),"",Y194-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE194="",'多次统计数据'!$B$8=""),"",AE194-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA194" s="10">
@@ -13949,6 +14729,10 @@
         <v/>
       </c>
       <c r="AD194" s="2" t="n"/>
+      <c r="AE194" s="7">
+        <f>IF(OR(X194="",C194="",C194&lt;=0),"",X194/C194)</f>
+        <v/>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="n"/>
@@ -14001,7 +14785,7 @@
         <v/>
       </c>
       <c r="Z195" s="7">
-        <f>IF(OR(Y195="",'多次统计数据'!$B$8=""),"",Y195-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE195="",'多次统计数据'!$B$8=""),"",AE195-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA195" s="10">
@@ -14017,6 +14801,10 @@
         <v/>
       </c>
       <c r="AD195" s="2" t="n"/>
+      <c r="AE195" s="7">
+        <f>IF(OR(X195="",C195="",C195&lt;=0),"",X195/C195)</f>
+        <v/>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="n"/>
@@ -14069,7 +14857,7 @@
         <v/>
       </c>
       <c r="Z196" s="7">
-        <f>IF(OR(Y196="",'多次统计数据'!$B$8=""),"",Y196-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE196="",'多次统计数据'!$B$8=""),"",AE196-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA196" s="10">
@@ -14085,6 +14873,10 @@
         <v/>
       </c>
       <c r="AD196" s="2" t="n"/>
+      <c r="AE196" s="7">
+        <f>IF(OR(X196="",C196="",C196&lt;=0),"",X196/C196)</f>
+        <v/>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="n"/>
@@ -14137,7 +14929,7 @@
         <v/>
       </c>
       <c r="Z197" s="7">
-        <f>IF(OR(Y197="",'多次统计数据'!$B$8=""),"",Y197-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE197="",'多次统计数据'!$B$8=""),"",AE197-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA197" s="10">
@@ -14153,6 +14945,10 @@
         <v/>
       </c>
       <c r="AD197" s="2" t="n"/>
+      <c r="AE197" s="7">
+        <f>IF(OR(X197="",C197="",C197&lt;=0),"",X197/C197)</f>
+        <v/>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="n"/>
@@ -14205,7 +15001,7 @@
         <v/>
       </c>
       <c r="Z198" s="7">
-        <f>IF(OR(Y198="",'多次统计数据'!$B$8=""),"",Y198-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE198="",'多次统计数据'!$B$8=""),"",AE198-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA198" s="10">
@@ -14221,6 +15017,10 @@
         <v/>
       </c>
       <c r="AD198" s="2" t="n"/>
+      <c r="AE198" s="7">
+        <f>IF(OR(X198="",C198="",C198&lt;=0),"",X198/C198)</f>
+        <v/>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="n"/>
@@ -14273,7 +15073,7 @@
         <v/>
       </c>
       <c r="Z199" s="7">
-        <f>IF(OR(Y199="",'多次统计数据'!$B$8=""),"",Y199-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE199="",'多次统计数据'!$B$8=""),"",AE199-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA199" s="10">
@@ -14289,6 +15089,10 @@
         <v/>
       </c>
       <c r="AD199" s="2" t="n"/>
+      <c r="AE199" s="7">
+        <f>IF(OR(X199="",C199="",C199&lt;=0),"",X199/C199)</f>
+        <v/>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="n"/>
@@ -14341,7 +15145,7 @@
         <v/>
       </c>
       <c r="Z200" s="7">
-        <f>IF(OR(Y200="",'多次统计数据'!$B$8=""),"",Y200-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE200="",'多次统计数据'!$B$8=""),"",AE200-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA200" s="10">
@@ -14357,6 +15161,10 @@
         <v/>
       </c>
       <c r="AD200" s="2" t="n"/>
+      <c r="AE200" s="7">
+        <f>IF(OR(X200="",C200="",C200&lt;=0),"",X200/C200)</f>
+        <v/>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="n"/>
@@ -14409,7 +15217,7 @@
         <v/>
       </c>
       <c r="Z201" s="7">
-        <f>IF(OR(Y201="",'多次统计数据'!$B$8=""),"",Y201-'多次统计数据'!$B$8)</f>
+        <f>IF(OR(AE201="",'多次统计数据'!$B$8=""),"",AE201-'多次统计数据'!$B$8)</f>
         <v/>
       </c>
       <c r="AA201" s="10">
@@ -14425,6 +15233,10 @@
         <v/>
       </c>
       <c r="AD201" s="2" t="n"/>
+      <c r="AE201" s="7">
+        <f>IF(OR(X201="",C201="",C201&lt;=0),"",X201/C201)</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="X2:X201">
@@ -14456,11 +15268,19 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="AE2:AE201">
+    <cfRule type="cellIs" priority="8" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="9" operator="lessThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="G2:G201">
-    <cfRule type="expression" priority="8" dxfId="1">
+    <cfRule type="expression" priority="10" dxfId="1">
       <formula>$G2="禁止开仓"</formula>
     </cfRule>
-    <cfRule type="expression" priority="9" dxfId="0">
+    <cfRule type="expression" priority="11" dxfId="0">
       <formula>$G2="允许开仓"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -20221,12 +21041,12 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>IFERROR(AVERAGEIF('单次交易'!X2:X201,"&gt;0",'单次交易'!Y2:Y201),"")</f>
+        <f>IFERROR(AVERAGEIF('单次交易'!X2:X201,"&gt;0",'单次交易'!AE2:AE201),"")</f>
         <v/>
       </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
-          <t>盈利交易实际收益率的平均值</t>
+          <t>盈利交易实际账户收益率的平均值</t>
         </is>
       </c>
     </row>
@@ -20237,12 +21057,12 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>IFERROR(-AVERAGEIF('单次交易'!X2:X201,"&lt;0",'单次交易'!Y2:Y201),"")</f>
+        <f>IFERROR(-AVERAGEIF('单次交易'!X2:X201,"&lt;0",'单次交易'!AE2:AE201),"")</f>
         <v/>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>以正数显示亏损幅度</t>
+          <t>亏损交易实际账户收益率绝对值的平均值</t>
         </is>
       </c>
     </row>
@@ -20317,12 +21137,12 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>IF(OR(B3+B4=0,B8="",B9=""),"",POWER(1+B8,B3)*POWER(1-B9,B4)-1)</f>
+        <f>IF(COUNT('单次交易'!AE2:AE201)=0,"",EXP(SUMPRODUCT(IFERROR(LN(1+'单次交易'!AE2:AE201),0)))-1)</f>
         <v/>
       </c>
       <c r="C14" s="12" t="inlineStr">
         <is>
-          <t>基于历史平均盈亏率的几何复利模拟</t>
+          <t>按每笔实际账户收益率逐笔连乘</t>
         </is>
       </c>
     </row>
@@ -20337,7 +21157,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -20498,6 +21318,22 @@
       <c r="C10" s="12" t="inlineStr">
         <is>
           <t>当月允许最大亏损金额－当前未平仓理论亏损</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>账户实际累计收益率</t>
+        </is>
+      </c>
+      <c r="B11" s="7">
+        <f>IF(OR(B2="",B3="",B2&lt;=0),"",B3/B2-1)</f>
+        <v/>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>当前总金额÷初始总金额－1；无入金出金时为账户权威累计收益</t>
         </is>
       </c>
     </row>
@@ -20642,12 +21478,12 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>IF(OR(B4="",B5="",B6="",B5&lt;=0,B6&lt;=0),"暂不可计算",ROUNDUP(B4/(B5*B6),0))</f>
+        <f>IF(OR(B3="",B6="",B3&lt;=0,B6&lt;=0),"暂不可计算",ROUNDUP(LN(1+B3)/LN(1+B6),0))</f>
         <v/>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>向上取整；历史期望收益率不为正时不计算</t>
+          <t>按目标收益率与历史账户期望收益率复利计算并向上取整</t>
         </is>
       </c>
     </row>

</xml_diff>